<commit_message>
Update budget: leave 1 June, £700 already spent, gym paid, £250 one-offs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Riu8Yf6aermiJMNVjCXVik
</commit_message>
<xml_diff>
--- a/Uni_Budget_2026-27.xlsx
+++ b/Uni_Budget_2026-27.xlsx
@@ -35,7 +35,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Assumption: mid-June 2027. Change this to the day you actually leave.</t>
+          <t xml:space="preserve">Assumption: around 1 June 2027 (your estimate). Change this to the day you actually leave.</t>
         </r>
       </text>
     </comment>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="112">
   <si>
     <t xml:space="preserve">Uni of Bath Budget: October 2026 to June 2027</t>
   </si>
@@ -142,6 +142,12 @@
     <t xml:space="preserve">Your figure: £24 a week.</t>
   </si>
   <si>
+    <t xml:space="preserve">Already spent before 5 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your figure: ~£700 spent in Sept/early Oct (includes the £400 gym and ~2.5 weeks of living costs).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total income</t>
   </si>
   <si>
@@ -235,16 +241,16 @@
     <t xml:space="preserve">Your figure. Check student plans and cancel anything you haven't used in a month.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gym membership</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Your figure: £400 for the year. If already paid, set to 0 and lower the SFE figure by what's already gone.</t>
+    <t xml:space="preserve">Gym membership (already paid)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£400 already paid, so it's counted in the 'Already spent' income row, not here.</t>
   </si>
   <si>
     <t xml:space="preserve">One-offs (Christmas gifts, books, haircuts, clothes)</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSUMPTION: £150 buffer for the year. Change it if you know your plans.</t>
+    <t xml:space="preserve">ASSUMPTION: £250 buffer for the year (you said maybe more than £150). Change it if you know your plans.</t>
   </si>
   <si>
     <t xml:space="preserve">Total spending</t>
@@ -337,28 +343,28 @@
     <t xml:space="preserve">THE BIG PICTURE</t>
   </si>
   <si>
-    <t xml:space="preserve">Your current habits use almost all of your income. Your lifestyle is affordable, but there's almost nothing spare for emergencies or savings. The Summary on the Budget tab shows the exact figures.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Suggested plan frees up about £45 a week (about £1,600 by June) without cutting anything completely.</t>
+    <t xml:space="preserve">Your current habits cost slightly MORE than you have, about £6.60 a week over, so you'd run short before June with nothing for emergencies or savings. The Summary on the Budget tab shows the exact figures.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Suggested plan frees up about £45 a week (about £1,575 by June) without cutting anything completely.</t>
   </si>
   <si>
     <t xml:space="preserve">BIGGEST WINS (ranked by money saved)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Groceries (£70 → £55): this is your biggest cost. Aldi and Lidl are usually much cheaper than Sainsbury's or Waitrose, and Bath has both. Batch-cook 2–3 meals on Sunday, plan meals before you shop and use own-brand. Saves about £540 by June.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Coffee (£21 → £9): £3 a day adds up to about £750 by June. A cafetière and a bag of decent coffee costs about £15 and lasts weeks. Keep bought coffee as a treat on 3 days. Saves about £430.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Nights out (£40 → £30): do pre-drinks, take a set amount of cash and leave your card at home, and look for SU or student-night deals. Saves about £360.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Takeaway (£15 → £10): collect instead of delivery (no fees), use student discount apps, or swap every other takeaway for a 'fakeaway' night. Saves about £180.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Laundry (£10 → £7): wash full loads only and skip the dryer by using a clothes airer (about £15). Saves about £110.</t>
+    <t xml:space="preserve">1. Groceries (£70 → £55): this is your biggest cost. Aldi and Lidl are usually much cheaper than Sainsbury's or Waitrose, and Bath has both. Batch-cook 2–3 meals on Sunday, plan meals before you shop and use own-brand. Saves about £525 by June.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Coffee (£21 → £9): £3 a day adds up to about £735 by June. A cafetière and a bag of decent coffee costs about £15 and lasts weeks. Keep bought coffee as a treat on 3 days. Saves about £420.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Nights out (£40 → £30): do pre-drinks, take a set amount of cash and leave your card at home, and look for SU or student-night deals. Saves about £350.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Takeaway (£15 → £10): collect instead of delivery (no fees), use student discount apps, or swap every other takeaway for a 'fakeaway' night. Saves about £175.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Laundry (£10 → £7): wash full loads only and skip the dryer by using a clothes airer (about £15). Saves about £105.</t>
   </si>
   <si>
     <t xml:space="preserve">HABITS THAT MAKE A BUDGET STICK</t>
@@ -385,7 +391,7 @@
     <t xml:space="preserve">• Check your subscriptions. Many have student or family plans, or can be shared.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Get the most from your £400 gym membership. If you go about 3 times a week it's under £3 a visit.</t>
+    <t xml:space="preserve">• You've already paid £400 for the gym, so use it. At about 3 visits a week it's under £3 a visit, and it's a free alternative to some nights out.</t>
   </si>
   <si>
     <t xml:space="preserve">SAFETY NET</t>
@@ -982,7 +988,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1025,7 +1031,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>46551</v>
+        <v>46539</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1033,8 +1039,8 @@
         <v>5</v>
       </c>
       <c r="B7" s="7" t="n">
-        <f aca="false">ROUND((B6-B5+1)/7,0)</f>
-        <v>36</v>
+        <f aca="false">ROUNDUP((B6-B5+1)/7,0)</f>
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1090,7 +1096,7 @@
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">IF($C13="Weekly",B13,IF($C13="Monthly",B13*12/52,B13/$B$7))</f>
-        <v>138.888888888889</v>
+        <v>142.857142857143</v>
       </c>
       <c r="E13" s="13" t="n">
         <f aca="false">D13*$B$7</f>
@@ -1112,7 +1118,7 @@
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">IF($C14="Weekly",B14,IF($C14="Monthly",B14*12/52,B14/$B$7))</f>
-        <v>27.7777777777778</v>
+        <v>28.5714285714286</v>
       </c>
       <c r="E14" s="13" t="n">
         <f aca="false">D14*$B$7</f>
@@ -1138,183 +1144,165 @@
       </c>
       <c r="E15" s="13" t="n">
         <f aca="false">D15*$B$7</f>
-        <v>864</v>
+        <v>840</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17" t="n">
-        <f aca="false">SUM(D13:D15)</f>
-        <v>190.666666666667</v>
-      </c>
-      <c r="E16" s="17" t="n">
-        <f aca="false">SUM(E13:E15)</f>
-        <v>6864</v>
-      </c>
-      <c r="F16" s="16"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="B16" s="12" t="n">
+        <v>-700</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <f aca="false">IF($C16="Weekly",B16,IF($C16="Monthly",B16*12/52,B16/$B$7))</f>
+        <v>-20</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <f aca="false">D16*$B$7</f>
+        <v>-700</v>
+      </c>
+      <c r="F16" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="17" t="n">
+        <f aca="false">SUM(D13:D16)</f>
+        <v>175.428571428571</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <f aca="false">SUM(E13:E16)</f>
+        <v>6140</v>
+      </c>
+      <c r="F17" s="16"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="10" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F19" s="10" t="s">
+      <c r="D20" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="E20" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="F20" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="G20" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="J19" s="10" t="s">
+      <c r="H20" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="K19" s="10" t="s">
+      <c r="I20" s="10" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+      <c r="J20" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="K20" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="12" t="n">
         <v>70</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D20" s="13" t="n">
-        <f aca="false">IF($C20="Weekly",B20,IF($C20="Monthly",B20*12/52,B20/$B$7))</f>
-        <v>70</v>
-      </c>
-      <c r="E20" s="13" t="n">
-        <f aca="false">D20*$B$7</f>
-        <v>2520</v>
-      </c>
-      <c r="F20" s="12" t="n">
-        <v>55</v>
-      </c>
-      <c r="G20" s="13" t="n">
-        <f aca="false">IF($C20="Weekly",F20,IF($C20="Monthly",F20*12/52,F20/$B$7))</f>
-        <v>55</v>
-      </c>
-      <c r="H20" s="13" t="n">
-        <f aca="false">G20*$B$7</f>
-        <v>1980</v>
-      </c>
-      <c r="I20" s="13" t="n">
-        <f aca="false">E20-H20</f>
-        <v>540</v>
-      </c>
-      <c r="J20" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="K20" s="18" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B21" s="12" t="n">
-        <v>10</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">IF($C21="Weekly",B21,IF($C21="Monthly",B21*12/52,B21/$B$7))</f>
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">D21*$B$7</f>
-        <v>360</v>
+        <v>2450</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">IF($C21="Weekly",F21,IF($C21="Monthly",F21*12/52,F21/$B$7))</f>
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="H21" s="13" t="n">
         <f aca="false">G21*$B$7</f>
-        <v>252</v>
+        <v>1925</v>
       </c>
       <c r="I21" s="13" t="n">
         <f aca="false">E21-H21</f>
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K21" s="18" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
         <v>41</v>
       </c>
       <c r="B22" s="12" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D22" s="13" t="n">
         <f aca="false">IF($C22="Weekly",B22,IF($C22="Monthly",B22*12/52,B22/$B$7))</f>
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E22" s="13" t="n">
         <f aca="false">D22*$B$7</f>
-        <v>756</v>
+        <v>350</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">IF($C22="Weekly",F22,IF($C22="Monthly",F22*12/52,F22/$B$7))</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H22" s="13" t="n">
         <f aca="false">G22*$B$7</f>
-        <v>324</v>
+        <v>245</v>
       </c>
       <c r="I22" s="13" t="n">
         <f aca="false">E22-H22</f>
-        <v>432</v>
+        <v>105</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K22" s="18" t="s">
         <v>42</v>
@@ -1325,36 +1313,36 @@
         <v>43</v>
       </c>
       <c r="B23" s="12" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="13" t="n">
         <f aca="false">IF($C23="Weekly",B23,IF($C23="Monthly",B23*12/52,B23/$B$7))</f>
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="E23" s="13" t="n">
         <f aca="false">D23*$B$7</f>
-        <v>1440</v>
+        <v>735</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">IF($C23="Weekly",F23,IF($C23="Monthly",F23*12/52,F23/$B$7))</f>
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H23" s="13" t="n">
         <f aca="false">G23*$B$7</f>
-        <v>1080</v>
+        <v>315</v>
       </c>
       <c r="I23" s="13" t="n">
         <f aca="false">E23-H23</f>
-        <v>360</v>
+        <v>420</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K23" s="18" t="s">
         <v>44</v>
@@ -1364,37 +1352,37 @@
       <c r="A24" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="8" t="n">
-        <v>15</v>
+      <c r="B24" s="12" t="n">
+        <v>40</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="13" t="n">
         <f aca="false">IF($C24="Weekly",B24,IF($C24="Monthly",B24*12/52,B24/$B$7))</f>
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="E24" s="13" t="n">
         <f aca="false">D24*$B$7</f>
-        <v>540</v>
-      </c>
-      <c r="F24" s="8" t="n">
-        <v>10</v>
+        <v>1400</v>
+      </c>
+      <c r="F24" s="12" t="n">
+        <v>30</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">IF($C24="Weekly",F24,IF($C24="Monthly",F24*12/52,F24/$B$7))</f>
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H24" s="13" t="n">
         <f aca="false">G24*$B$7</f>
-        <v>360</v>
+        <v>1050</v>
       </c>
       <c r="I24" s="13" t="n">
         <f aca="false">E24-H24</f>
-        <v>180</v>
+        <v>350</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K24" s="18" t="s">
         <v>46</v>
@@ -1404,77 +1392,77 @@
       <c r="A25" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B25" s="12" t="n">
-        <v>12.5</v>
+      <c r="B25" s="8" t="n">
+        <v>15</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="13" t="n">
         <f aca="false">IF($C25="Weekly",B25,IF($C25="Monthly",B25*12/52,B25/$B$7))</f>
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="E25" s="13" t="n">
         <f aca="false">D25*$B$7</f>
-        <v>450</v>
-      </c>
-      <c r="F25" s="12" t="n">
-        <v>12.5</v>
+        <v>525</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>10</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">IF($C25="Weekly",F25,IF($C25="Monthly",F25*12/52,F25/$B$7))</f>
-        <v>12.5</v>
+        <v>10</v>
       </c>
       <c r="H25" s="13" t="n">
         <f aca="false">G25*$B$7</f>
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="I25" s="13" t="n">
         <f aca="false">E25-H25</f>
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K25" s="18" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="8" t="n">
-        <v>5</v>
+      <c r="B26" s="12" t="n">
+        <v>12.5</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="13" t="n">
         <f aca="false">IF($C26="Weekly",B26,IF($C26="Monthly",B26*12/52,B26/$B$7))</f>
-        <v>5</v>
+        <v>12.5</v>
       </c>
       <c r="E26" s="13" t="n">
         <f aca="false">D26*$B$7</f>
-        <v>180</v>
-      </c>
-      <c r="F26" s="8" t="n">
-        <v>5</v>
+        <v>437.5</v>
+      </c>
+      <c r="F26" s="12" t="n">
+        <v>12.5</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">IF($C26="Weekly",F26,IF($C26="Monthly",F26*12/52,F26/$B$7))</f>
-        <v>5</v>
+        <v>12.5</v>
       </c>
       <c r="H26" s="13" t="n">
         <f aca="false">G26*$B$7</f>
-        <v>180</v>
+        <v>437.5</v>
       </c>
       <c r="I26" s="13" t="n">
         <f aca="false">E26-H26</f>
         <v>0</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K26" s="18" t="s">
         <v>50</v>
@@ -1484,77 +1472,77 @@
       <c r="A27" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="12" t="n">
-        <v>6</v>
+      <c r="B27" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="D27" s="13" t="n">
         <f aca="false">IF($C27="Weekly",B27,IF($C27="Monthly",B27*12/52,B27/$B$7))</f>
-        <v>1.38461538461538</v>
+        <v>5</v>
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">D27*$B$7</f>
-        <v>49.8461538461539</v>
-      </c>
-      <c r="F27" s="12" t="n">
-        <v>6</v>
+        <v>175</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">IF($C27="Weekly",F27,IF($C27="Monthly",F27*12/52,F27/$B$7))</f>
-        <v>1.38461538461538</v>
+        <v>5</v>
       </c>
       <c r="H27" s="13" t="n">
         <f aca="false">G27*$B$7</f>
-        <v>49.8461538461539</v>
+        <v>175</v>
       </c>
       <c r="I27" s="13" t="n">
         <f aca="false">E27-H27</f>
         <v>0</v>
       </c>
       <c r="J27" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="K27" s="18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="K27" s="18" t="s">
+      <c r="B28" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B28" s="12" t="n">
-        <v>400</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>17</v>
       </c>
       <c r="D28" s="13" t="n">
         <f aca="false">IF($C28="Weekly",B28,IF($C28="Monthly",B28*12/52,B28/$B$7))</f>
-        <v>11.1111111111111</v>
+        <v>1.38461538461538</v>
       </c>
       <c r="E28" s="13" t="n">
         <f aca="false">D28*$B$7</f>
-        <v>400</v>
+        <v>48.4615384615385</v>
       </c>
       <c r="F28" s="12" t="n">
-        <v>400</v>
+        <v>6</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">IF($C28="Weekly",F28,IF($C28="Monthly",F28*12/52,F28/$B$7))</f>
-        <v>11.1111111111111</v>
+        <v>1.38461538461538</v>
       </c>
       <c r="H28" s="13" t="n">
         <f aca="false">G28*$B$7</f>
-        <v>400</v>
+        <v>48.4615384615385</v>
       </c>
       <c r="I28" s="13" t="n">
         <f aca="false">E28-H28</f>
         <v>0</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="K28" s="18" t="s">
         <v>56</v>
@@ -1564,192 +1552,232 @@
       <c r="A29" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="8" t="n">
-        <v>150</v>
+      <c r="B29" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D29" s="13" t="n">
         <f aca="false">IF($C29="Weekly",B29,IF($C29="Monthly",B29*12/52,B29/$B$7))</f>
-        <v>4.16666666666667</v>
+        <v>0</v>
       </c>
       <c r="E29" s="13" t="n">
         <f aca="false">D29*$B$7</f>
-        <v>150</v>
-      </c>
-      <c r="F29" s="8" t="n">
-        <v>150</v>
+        <v>0</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">IF($C29="Weekly",F29,IF($C29="Monthly",F29*12/52,F29/$B$7))</f>
-        <v>4.16666666666667</v>
+        <v>0</v>
       </c>
       <c r="H29" s="13" t="n">
         <f aca="false">G29*$B$7</f>
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="I29" s="13" t="n">
         <f aca="false">E29-H29</f>
         <v>0</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="K29" s="18" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="17" t="n">
-        <f aca="false">SUM(D20:D29)</f>
-        <v>190.162393162393</v>
-      </c>
-      <c r="E30" s="17" t="n">
-        <f aca="false">SUM(E20:E29)</f>
-        <v>6845.84615384615</v>
-      </c>
-      <c r="F30" s="16"/>
-      <c r="G30" s="17" t="n">
-        <f aca="false">SUM(G20:G29)</f>
-        <v>145.162393162393</v>
-      </c>
-      <c r="H30" s="17" t="n">
-        <f aca="false">SUM(H20:H29)</f>
-        <v>5225.84615384615</v>
-      </c>
-      <c r="I30" s="17" t="n">
-        <f aca="false">SUM(I20:I29)</f>
-        <v>1620</v>
-      </c>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="B30" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="13" t="n">
+        <f aca="false">IF($C30="Weekly",B30,IF($C30="Monthly",B30*12/52,B30/$B$7))</f>
+        <v>7.14285714285714</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <f aca="false">D30*$B$7</f>
+        <v>250</v>
+      </c>
+      <c r="F30" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="G30" s="13" t="n">
+        <f aca="false">IF($C30="Weekly",F30,IF($C30="Monthly",F30*12/52,F30/$B$7))</f>
+        <v>7.14285714285714</v>
+      </c>
+      <c r="H30" s="13" t="n">
+        <f aca="false">G30*$B$7</f>
+        <v>250</v>
+      </c>
+      <c r="I30" s="13" t="n">
+        <f aca="false">E30-H30</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="K30" s="18" t="s">
         <v>60</v>
       </c>
     </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="17" t="n">
+        <f aca="false">SUM(D21:D30)</f>
+        <v>182.027472527473</v>
+      </c>
+      <c r="E31" s="17" t="n">
+        <f aca="false">SUM(E21:E30)</f>
+        <v>6370.96153846154</v>
+      </c>
+      <c r="F31" s="16"/>
+      <c r="G31" s="17" t="n">
+        <f aca="false">SUM(G21:G30)</f>
+        <v>137.027472527473</v>
+      </c>
+      <c r="H31" s="17" t="n">
+        <f aca="false">SUM(H21:H30)</f>
+        <v>4795.96153846154</v>
+      </c>
+      <c r="I31" s="17" t="n">
+        <f aca="false">SUM(I21:I30)</f>
+        <v>1575</v>
+      </c>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+    </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" s="10" t="s">
+      <c r="A33" s="3" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="10"/>
+      <c r="B34" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B34" s="19" t="n">
-        <f aca="false">$D$16</f>
-        <v>190.666666666667</v>
-      </c>
-      <c r="C34" s="19" t="n">
-        <f aca="false">$D$16</f>
-        <v>190.666666666667</v>
+      <c r="C34" s="10" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B35" s="13" t="n">
-        <f aca="false">D30</f>
-        <v>190.162393162393</v>
-      </c>
-      <c r="C35" s="13" t="n">
-        <f aca="false">G30</f>
-        <v>145.162393162393</v>
+        <v>65</v>
+      </c>
+      <c r="B35" s="19" t="n">
+        <f aca="false">$D$17</f>
+        <v>175.428571428571</v>
+      </c>
+      <c r="C35" s="19" t="n">
+        <f aca="false">$D$17</f>
+        <v>175.428571428571</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B36" s="13" t="n">
-        <f aca="false">B34-B35</f>
-        <v>0.504273504273499</v>
+        <f aca="false">D31</f>
+        <v>182.027472527473</v>
       </c>
       <c r="C36" s="13" t="n">
-        <f aca="false">C34-C35</f>
-        <v>45.5042735042735</v>
+        <f aca="false">G31</f>
+        <v>137.027472527473</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B37" s="19" t="n">
+        <v>67</v>
+      </c>
+      <c r="B37" s="13" t="n">
+        <f aca="false">B35-B36</f>
+        <v>-6.59890109890108</v>
+      </c>
+      <c r="C37" s="13" t="n">
+        <f aca="false">C35-C36</f>
+        <v>38.4010989010989</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" s="19" t="n">
         <f aca="false">$B$8</f>
         <v>25</v>
       </c>
-      <c r="C37" s="19" t="n">
+      <c r="C38" s="19" t="n">
         <f aca="false">$B$8</f>
         <v>25</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B38" s="13" t="n">
-        <f aca="false">B36-B37</f>
-        <v>-24.4957264957265</v>
-      </c>
-      <c r="C38" s="13" t="n">
-        <f aca="false">C36-C37</f>
-        <v>20.5042735042735</v>
-      </c>
-    </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B39" s="13" t="n">
-        <f aca="false">B36*$B$7</f>
-        <v>18.153846153846</v>
+        <f aca="false">B37-B38</f>
+        <v>-31.5989010989011</v>
       </c>
       <c r="C39" s="13" t="n">
-        <f aca="false">C36*$B$7</f>
-        <v>1638.15384615385</v>
+        <f aca="false">C37-C38</f>
+        <v>13.4010989010989</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B40" s="13" t="n">
-        <f aca="false">MAX(0,MIN(B36,$B$8))*$B$7</f>
-        <v>18.153846153846</v>
+        <f aca="false">B37*$B$7</f>
+        <v>-230.961538461538</v>
       </c>
       <c r="C40" s="13" t="n">
-        <f aca="false">MAX(0,MIN(C36,$B$8))*$B$7</f>
-        <v>900</v>
+        <f aca="false">C37*$B$7</f>
+        <v>1344.03846153846</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B41" s="4" t="str">
-        <f aca="false">IF(B38&gt;=0,"On track",IF(B36&gt;=0,"Can't hit savings target","Overspending"))</f>
-        <v>Can't hit savings target</v>
-      </c>
-      <c r="C41" s="4" t="str">
-        <f aca="false">IF(C38&gt;=0,"On track",IF(C36&gt;=0,"Can't hit savings target","Overspending"))</f>
+        <v>71</v>
+      </c>
+      <c r="B41" s="13" t="n">
+        <f aca="false">MAX(0,MIN(B37,$B$8))*$B$7</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="13" t="n">
+        <f aca="false">MAX(0,MIN(C37,$B$8))*$B$7</f>
+        <v>875</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B42" s="4" t="str">
+        <f aca="false">IF(B39&gt;=0,"On track",IF(B37&gt;=0,"Can't hit savings target","Overspending"))</f>
+        <v>Overspending</v>
+      </c>
+      <c r="C42" s="4" t="str">
+        <f aca="false">IF(C39&gt;=0,"On track",IF(C37&gt;=0,"Can't hit savings target","Overspending"))</f>
         <v>On track</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B41:C41">
+  <conditionalFormatting sqref="B42:C42">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"On track"</formula>
     </cfRule>
@@ -1757,7 +1785,7 @@
       <formula>"On track"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B36:C38">
+  <conditionalFormatting sqref="B37:C39">
     <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -1767,7 +1795,7 @@
       <formula1>"Suggested,Current"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C13:C15 C20:C29" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C13:C16 C21:C30" type="list">
       <formula1>"Weekly,Monthly,Per period"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1798,42 +1826,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10"/>
       <c r="B4" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K4" s="10"/>
       <c r="L4" s="10"/>
@@ -1845,31 +1873,31 @@
         <v>Plan: Suggested</v>
       </c>
       <c r="C5" s="19" t="n">
-        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$20,Budget!$G$20)</f>
+        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$21,Budget!$G$21)</f>
         <v>55</v>
       </c>
       <c r="D5" s="19" t="n">
-        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$21,Budget!$G$21)</f>
+        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$22,Budget!$G$22)</f>
         <v>7</v>
       </c>
       <c r="E5" s="19" t="n">
-        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$22,Budget!$G$22)</f>
+        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$23,Budget!$G$23)</f>
         <v>9</v>
       </c>
       <c r="F5" s="19" t="n">
-        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$23,Budget!$G$23)</f>
+        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$24,Budget!$G$24)</f>
         <v>30</v>
       </c>
       <c r="G5" s="19" t="n">
-        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$24,Budget!$G$24)</f>
+        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$25,Budget!$G$25)</f>
         <v>10</v>
       </c>
       <c r="H5" s="19" t="n">
-        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$25,Budget!$G$25)</f>
+        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$26,Budget!$G$26)</f>
         <v>12.5</v>
       </c>
       <c r="I5" s="19" t="n">
-        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$26,Budget!$G$26)</f>
+        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$27,Budget!$G$27)</f>
         <v>5</v>
       </c>
       <c r="J5" s="21" t="n">
@@ -1879,10 +1907,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>52.3</v>
@@ -1921,43 +1949,43 @@
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3084,9 +3112,9 @@
       <c r="A45" s="11" t="n">
         <v>36</v>
       </c>
-      <c r="B45" s="25" t="n">
+      <c r="B45" s="25" t="str">
         <f aca="false">IF(A45&gt;Budget!$B$7,"",Budget!$B$5+(A45-1)*7)</f>
-        <v>46545</v>
+        <v/>
       </c>
       <c r="C45" s="12"/>
       <c r="D45" s="12"/>
@@ -3099,9 +3127,9 @@
         <f aca="false">IF(COUNT(C45:I45)=0,"",SUM(C45:I45))</f>
         <v/>
       </c>
-      <c r="K45" s="13" t="n">
+      <c r="K45" s="13" t="str">
         <f aca="false">IF(B45="","",$J$5)</f>
-        <v>128.5</v>
+        <v/>
       </c>
       <c r="L45" s="13" t="str">
         <f aca="false">IF(J45="","",K45-J45)</f>
@@ -3242,7 +3270,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="15" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B50" s="16"/>
       <c r="C50" s="17" t="n">
@@ -3286,7 +3314,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B51" s="16"/>
       <c r="C51" s="17" t="str">
@@ -3370,22 +3398,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="27" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3393,32 +3421,32 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3426,47 +3454,47 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="27" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3474,22 +3502,22 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="26" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="27" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebalance budget to spend everything by 1 June
Savings target set to 0, suggested plan adjusted, and a calculated
Flexible / treats row keeps the plan balanced at exactly zero.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Riu8Yf6aermiJMNVjCXVik
</commit_message>
<xml_diff>
--- a/Uni_Budget_2026-27.xlsx
+++ b/Uni_Budget_2026-27.xlsx
@@ -47,7 +47,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Suggested target: £25/week is about £900 by June. Only reachable with the 'Suggested' plan.</t>
+          <t xml:space="preserve">Suggested target: set to 0 because you asked to finish with nothing spare in June. Raise it to save; the Flexible row shrinks to match.</t>
         </r>
       </text>
     </comment>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="116">
   <si>
     <t xml:space="preserve">Uni of Bath Budget: October 2026 to June 2027</t>
   </si>
@@ -199,10 +199,10 @@
     <t xml:space="preserve">Wash only full loads and dry on a clothes airer instead of the tumble dryer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Coffee (£3 x 7 days)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Have 3 bought coffees a week and make the rest at home or in halls. Bring a reusable cup for discounts.</t>
+    <t xml:space="preserve">Coffee (£3 a day)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan: 6 bought coffees a week. Make 1 at home and bring a reusable cup for discounts.</t>
   </si>
   <si>
     <t xml:space="preserve">Nights out (2 x £20)</t>
@@ -253,6 +253,12 @@
     <t xml:space="preserve">ASSUMPTION: £250 buffer for the year (you said maybe more than £150). Change it if you know your plans.</t>
   </si>
   <si>
+    <t xml:space="preserve">Flexible / treats (balancing figure)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculated automatically: whatever is left after everything else and your savings target, so you finish June on £0. If it goes red (negative), cut something above.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total spending</t>
   </si>
   <si>
@@ -307,6 +313,9 @@
     <t xml:space="preserve">Takeaway</t>
   </si>
   <si>
+    <t xml:space="preserve">Flexible / treats</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
@@ -343,43 +352,43 @@
     <t xml:space="preserve">THE BIG PICTURE</t>
   </si>
   <si>
-    <t xml:space="preserve">Your current habits cost slightly MORE than you have, about £6.60 a week over, so you'd run short before June with nothing for emergencies or savings. The Summary on the Budget tab shows the exact figures.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Suggested plan frees up about £45 a week (about £1,575 by June) without cutting anything completely.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIGGEST WINS (ranked by money saved)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Groceries (£70 → £55): this is your biggest cost. Aldi and Lidl are usually much cheaper than Sainsbury's or Waitrose, and Bath has both. Batch-cook 2–3 meals on Sunday, plan meals before you shop and use own-brand. Saves about £525 by June.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Coffee (£21 → £9): £3 a day adds up to about £735 by June. A cafetière and a bag of decent coffee costs about £15 and lasts weeks. Keep bought coffee as a treat on 3 days. Saves about £420.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Nights out (£40 → £30): do pre-drinks, take a set amount of cash and leave your card at home, and look for SU or student-night deals. Saves about £350.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Takeaway (£15 → £10): collect instead of delivery (no fees), use student discount apps, or swap every other takeaway for a 'fakeaway' night. Saves about £175.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Laundry (£10 → £7): wash full loads only and skip the dryer by using a clothes airer (about £15). Saves about £105.</t>
+    <t xml:space="preserve">This plan spends every penny: you finish on £0 when you leave on 1 June. The 'Flexible / treats' row on the Budget tab is calculated automatically, so the plan always balances to exactly £0, even if you change other numbers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your current habits cost about £6.60 a week more than you have (about £230 short by June). The plan closes that gap with three small changes and keeps your nights out and takeaways as they are.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THE THREE SMALL CHANGES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Groceries (£70 → £65): shop at Aldi or Lidl for the basics and use own-brand. Saves about £175 by June.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Coffee (£21 → £18): six bought coffees a week instead of seven, and make one at home. Saves about £105.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Laundry (£10 → £8): wash full loads only and use a clothes airer instead of the dryer. Saves about £70.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IF YOU WANT MORE BREATHING ROOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Every £1 a week you cut from anything above adds £1 a week to 'Flexible / treats' (about £35 by June).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Easy extras: buy 3 coffees a week instead of 6 (+£9/week), do pre-drinks before nights out (+£5–10/week), collect takeaways instead of delivery (+£3/week).</t>
   </si>
   <si>
     <t xml:space="preserve">HABITS THAT MAKE A BUDGET STICK</t>
   </si>
   <si>
-    <t xml:space="preserve">• Pay yourself first. When money comes in (each SFE instalment, the grandparents' money), move your savings target into a separate savings pot straight away.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Use a 'spending pot'. Many banking apps (Monzo, Starling, etc.) let you set up pots. Move your weekly limit into a spending pot every Monday and spend only from that.</t>
+    <t xml:space="preserve">• Use a 'spending pot'. Many banking apps (Monzo, Starling, etc.) let you set up pots. Move your weekly limit from the Weekly Tracker into a spending pot every Monday and spend only from that.</t>
   </si>
   <si>
     <t xml:space="preserve">• Take 5 minutes every Sunday to fill in the Weekly Tracker. Red cells show where the money is going.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Spread out big payments. Your SFE comes in 3 lumps, so don't treat payday week as 'rich week'. The weekly figure on the Budget tab is what you can really spend.</t>
+    <t xml:space="preserve">• Spread out big payments. Your SFE comes in 3 lumps, so don't treat payday week as 'rich week'. The weekly figure is what you can really spend.</t>
   </si>
   <si>
     <t xml:space="preserve">• Plan for January. The first instalment has to last until the second, and Christmas is in between. Keep an eye on the running total in the Tracker.</t>
@@ -391,13 +400,16 @@
     <t xml:space="preserve">• Check your subscriptions. Many have student or family plans, or can be shared.</t>
   </si>
   <si>
-    <t xml:space="preserve">• You've already paid £400 for the gym, so use it. At about 3 visits a week it's under £3 a visit, and it's a free alternative to some nights out.</t>
+    <t xml:space="preserve">• You've already paid £400 for the gym, so use it. It's a free alternative to some nights out.</t>
   </si>
   <si>
     <t xml:space="preserve">SAFETY NET</t>
   </si>
   <si>
-    <t xml:space="preserve">• Aim to keep a £200–£300 emergency buffer that you don't touch, for things like a broken phone or an unexpected trip home.</t>
+    <t xml:space="preserve">• Spending down to £0 means there's no cushion for surprises. The £250 one-offs buffer is the nearest thing to one, so try not to use it all before May.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• If you go over one week, spend less the next week. The running total in the Tracker should stay at or above £0.</t>
   </si>
   <si>
     <t xml:space="preserve">• If money gets tight, the University of Bath Student Money Advice team and the SU Advice service can help, including with hardship funds. Talk to them early, not when you're already in trouble.</t>
@@ -526,7 +538,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -549,6 +561,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
         <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -607,7 +625,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -684,6 +702,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -696,15 +718,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -733,14 +755,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -988,7 +1010,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1048,7 +1070,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1247,19 +1269,19 @@
         <v>2450</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">IF($C21="Weekly",F21,IF($C21="Monthly",F21*12/52,F21/$B$7))</f>
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H21" s="13" t="n">
         <f aca="false">G21*$B$7</f>
-        <v>1925</v>
+        <v>2275</v>
       </c>
       <c r="I21" s="13" t="n">
         <f aca="false">E21-H21</f>
-        <v>525</v>
+        <v>175</v>
       </c>
       <c r="J21" s="11" t="s">
         <v>39</v>
@@ -1287,19 +1309,19 @@
         <v>350</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">IF($C22="Weekly",F22,IF($C22="Monthly",F22*12/52,F22/$B$7))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H22" s="13" t="n">
         <f aca="false">G22*$B$7</f>
-        <v>245</v>
+        <v>280</v>
       </c>
       <c r="I22" s="13" t="n">
         <f aca="false">E22-H22</f>
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="J22" s="11" t="s">
         <v>39</v>
@@ -1308,7 +1330,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
         <v>43</v>
       </c>
@@ -1327,19 +1349,19 @@
         <v>735</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">IF($C23="Weekly",F23,IF($C23="Monthly",F23*12/52,F23/$B$7))</f>
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H23" s="13" t="n">
         <f aca="false">G23*$B$7</f>
-        <v>315</v>
+        <v>630</v>
       </c>
       <c r="I23" s="13" t="n">
         <f aca="false">E23-H23</f>
-        <v>420</v>
+        <v>105</v>
       </c>
       <c r="J23" s="11" t="s">
         <v>39</v>
@@ -1367,19 +1389,19 @@
         <v>1400</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">IF($C24="Weekly",F24,IF($C24="Monthly",F24*12/52,F24/$B$7))</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H24" s="13" t="n">
         <f aca="false">G24*$B$7</f>
-        <v>1050</v>
+        <v>1400</v>
       </c>
       <c r="I24" s="13" t="n">
         <f aca="false">E24-H24</f>
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="J24" s="11" t="s">
         <v>39</v>
@@ -1407,19 +1429,19 @@
         <v>525</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">IF($C25="Weekly",F25,IF($C25="Monthly",F25*12/52,F25/$B$7))</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H25" s="13" t="n">
         <f aca="false">G25*$B$7</f>
-        <v>350</v>
+        <v>525</v>
       </c>
       <c r="I25" s="13" t="n">
         <f aca="false">E25-H25</f>
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="J25" s="11" t="s">
         <v>39</v>
@@ -1628,165 +1650,211 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="17" t="n">
-        <f aca="false">SUM(D21:D30)</f>
+      <c r="B31" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D31" s="13" t="n">
+        <f aca="false">IF($C31="Weekly",B31,IF($C31="Monthly",B31*12/52,B31/$B$7))</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <f aca="false">D31*$B$7</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="19" t="n">
+        <f aca="false">ROUND($D$17-$B$8-SUM(G21:G30),2)</f>
+        <v>3.4</v>
+      </c>
+      <c r="G31" s="13" t="n">
+        <f aca="false">IF($C31="Weekly",F31,IF($C31="Monthly",F31*12/52,F31/$B$7))</f>
+        <v>3.4</v>
+      </c>
+      <c r="H31" s="13" t="n">
+        <f aca="false">G31*$B$7</f>
+        <v>119</v>
+      </c>
+      <c r="I31" s="13" t="n">
+        <f aca="false">E31-H31</f>
+        <v>-119</v>
+      </c>
+      <c r="J31" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="17" t="n">
+        <f aca="false">SUM(D21:D31)</f>
         <v>182.027472527473</v>
       </c>
-      <c r="E31" s="17" t="n">
-        <f aca="false">SUM(E21:E30)</f>
+      <c r="E32" s="17" t="n">
+        <f aca="false">SUM(E21:E31)</f>
         <v>6370.96153846154</v>
       </c>
-      <c r="F31" s="16"/>
-      <c r="G31" s="17" t="n">
-        <f aca="false">SUM(G21:G30)</f>
-        <v>137.027472527473</v>
-      </c>
-      <c r="H31" s="17" t="n">
-        <f aca="false">SUM(H21:H30)</f>
-        <v>4795.96153846154</v>
-      </c>
-      <c r="I31" s="17" t="n">
-        <f aca="false">SUM(I21:I30)</f>
-        <v>1575</v>
-      </c>
-      <c r="J31" s="16"/>
-      <c r="K31" s="16"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>62</v>
-      </c>
+      <c r="F32" s="16"/>
+      <c r="G32" s="17" t="n">
+        <f aca="false">SUM(G21:G31)</f>
+        <v>175.427472527473</v>
+      </c>
+      <c r="H32" s="17" t="n">
+        <f aca="false">SUM(H21:H31)</f>
+        <v>6139.96153846154</v>
+      </c>
+      <c r="I32" s="17" t="n">
+        <f aca="false">SUM(I21:I31)</f>
+        <v>231</v>
+      </c>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C34" s="10" t="s">
+      <c r="A34" s="3" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="10"/>
+      <c r="B35" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B35" s="19" t="n">
+      <c r="C35" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36" s="20" t="n">
         <f aca="false">$D$17</f>
         <v>175.428571428571</v>
       </c>
-      <c r="C35" s="19" t="n">
+      <c r="C36" s="20" t="n">
         <f aca="false">$D$17</f>
         <v>175.428571428571</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B36" s="13" t="n">
-        <f aca="false">D31</f>
-        <v>182.027472527473</v>
-      </c>
-      <c r="C36" s="13" t="n">
-        <f aca="false">G31</f>
-        <v>137.027472527473</v>
-      </c>
-    </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B37" s="13" t="n">
-        <f aca="false">B35-B36</f>
-        <v>-6.59890109890108</v>
+        <f aca="false">D32</f>
+        <v>182.027472527473</v>
       </c>
       <c r="C37" s="13" t="n">
-        <f aca="false">C35-C36</f>
-        <v>38.4010989010989</v>
+        <f aca="false">G32</f>
+        <v>175.427472527473</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B38" s="19" t="n">
-        <f aca="false">$B$8</f>
-        <v>25</v>
-      </c>
-      <c r="C38" s="19" t="n">
-        <f aca="false">$B$8</f>
-        <v>25</v>
+        <v>69</v>
+      </c>
+      <c r="B38" s="13" t="n">
+        <f aca="false">ROUND(B36-B37,2)</f>
+        <v>-6.6</v>
+      </c>
+      <c r="C38" s="13" t="n">
+        <f aca="false">ROUND(C36-C37,2)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B39" s="13" t="n">
-        <f aca="false">B37-B38</f>
-        <v>-31.5989010989011</v>
-      </c>
-      <c r="C39" s="13" t="n">
-        <f aca="false">C37-C38</f>
-        <v>13.4010989010989</v>
+        <v>70</v>
+      </c>
+      <c r="B39" s="20" t="n">
+        <f aca="false">$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="20" t="n">
+        <f aca="false">$B$8</f>
+        <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B40" s="13" t="n">
-        <f aca="false">B37*$B$7</f>
-        <v>-230.961538461538</v>
+        <f aca="false">ROUND(B38-B39,2)</f>
+        <v>-6.6</v>
       </c>
       <c r="C40" s="13" t="n">
-        <f aca="false">C37*$B$7</f>
-        <v>1344.03846153846</v>
+        <f aca="false">ROUND(C38-C39,2)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B41" s="13" t="n">
-        <f aca="false">MAX(0,MIN(B37,$B$8))*$B$7</f>
+        <f aca="false">B38*$B$7</f>
+        <v>-231</v>
+      </c>
+      <c r="C41" s="13" t="n">
+        <f aca="false">C38*$B$7</f>
         <v>0</v>
-      </c>
-      <c r="C41" s="13" t="n">
-        <f aca="false">MAX(0,MIN(C37,$B$8))*$B$7</f>
-        <v>875</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B42" s="4" t="str">
-        <f aca="false">IF(B39&gt;=0,"On track",IF(B37&gt;=0,"Can't hit savings target","Overspending"))</f>
+        <v>73</v>
+      </c>
+      <c r="B42" s="13" t="n">
+        <f aca="false">MAX(0,MIN(B38,$B$8))*$B$7</f>
+        <v>0</v>
+      </c>
+      <c r="C42" s="13" t="n">
+        <f aca="false">MAX(0,MIN(C38,$B$8))*$B$7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B43" s="4" t="str">
+        <f aca="false">IF(B40&gt;=0,"On track",IF(B38&gt;=0,"Can't hit savings target","Overspending"))</f>
         <v>Overspending</v>
       </c>
-      <c r="C42" s="4" t="str">
-        <f aca="false">IF(C39&gt;=0,"On track",IF(C37&gt;=0,"Can't hit savings target","Overspending"))</f>
+      <c r="C43" s="4" t="str">
+        <f aca="false">IF(C40&gt;=0,"On track",IF(C38&gt;=0,"Can't hit savings target","Overspending"))</f>
         <v>On track</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B42:C42">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+  <conditionalFormatting sqref="F31:H31">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B43:C43">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"On track"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="notEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="4" operator="notEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"On track"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B37:C39">
-    <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+  <conditionalFormatting sqref="B38:C40">
+    <cfRule type="cellIs" priority="5" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1795,7 +1863,7 @@
       <formula1>"Suggested,Current"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C13:C16 C21:C30" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C13:C16 C21:C31" type="list">
       <formula1>"Weekly,Monthly,Per period"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1816,28 +1884,28 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="3" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10"/>
       <c r="B4" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>38</v>
@@ -1846,13 +1914,13 @@
         <v>41</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>49</v>
@@ -1861,98 +1929,108 @@
         <v>51</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="K4" s="10"/>
+        <v>81</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>82</v>
+      </c>
       <c r="L4" s="10"/>
       <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="20" t="str">
+      <c r="B5" s="21" t="str">
         <f aca="false">"Plan: "&amp;Budget!$B$9</f>
         <v>Plan: Suggested</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="20" t="n">
         <f aca="false">IF(Budget!$B$9="Current",Budget!$D$21,Budget!$G$21)</f>
-        <v>55</v>
-      </c>
-      <c r="D5" s="19" t="n">
+        <v>65</v>
+      </c>
+      <c r="D5" s="20" t="n">
         <f aca="false">IF(Budget!$B$9="Current",Budget!$D$22,Budget!$G$22)</f>
-        <v>7</v>
-      </c>
-      <c r="E5" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" s="20" t="n">
         <f aca="false">IF(Budget!$B$9="Current",Budget!$D$23,Budget!$G$23)</f>
-        <v>9</v>
-      </c>
-      <c r="F5" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" s="20" t="n">
         <f aca="false">IF(Budget!$B$9="Current",Budget!$D$24,Budget!$G$24)</f>
-        <v>30</v>
-      </c>
-      <c r="G5" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="G5" s="20" t="n">
         <f aca="false">IF(Budget!$B$9="Current",Budget!$D$25,Budget!$G$25)</f>
-        <v>10</v>
-      </c>
-      <c r="H5" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H5" s="20" t="n">
         <f aca="false">IF(Budget!$B$9="Current",Budget!$D$26,Budget!$G$26)</f>
         <v>12.5</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="20" t="n">
         <f aca="false">IF(Budget!$B$9="Current",Budget!$D$27,Budget!$G$27)</f>
         <v>5</v>
       </c>
-      <c r="J5" s="21" t="n">
-        <f aca="false">SUM(C5:I5)</f>
-        <v>128.5</v>
+      <c r="J5" s="20" t="n">
+        <f aca="false">IF(Budget!$B$9="Current",Budget!$D$31,Budget!$G$31)</f>
+        <v>3.4</v>
+      </c>
+      <c r="K5" s="22" t="n">
+        <f aca="false">SUM(C5:J5)</f>
+        <v>166.9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="C7" s="23" t="n">
-        <v>52.3</v>
-      </c>
-      <c r="D7" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="E7" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="F7" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="G7" s="23" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="H7" s="23" t="n">
+      <c r="A7" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="24" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>38</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H7" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="I7" s="23" t="n">
+      <c r="I7" s="24" t="n">
         <v>3.2</v>
       </c>
-      <c r="J7" s="23" t="n">
-        <f aca="false">SUM(C7:I7)</f>
-        <v>130</v>
-      </c>
-      <c r="K7" s="23" t="n">
-        <f aca="false">$J$5</f>
-        <v>128.5</v>
-      </c>
-      <c r="L7" s="23" t="n">
-        <f aca="false">K7-J7</f>
-        <v>-1.5</v>
-      </c>
-      <c r="M7" s="24"/>
+      <c r="J7" s="24" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K7" s="24" t="n">
+        <f aca="false">SUM(C7:J7)</f>
+        <v>153.5</v>
+      </c>
+      <c r="L7" s="24" t="n">
+        <f aca="false">$K$5</f>
+        <v>166.9</v>
+      </c>
+      <c r="M7" s="24" t="n">
+        <f aca="false">L7-K7</f>
+        <v>13.4</v>
+      </c>
+      <c r="N7" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>38</v>
@@ -1961,13 +2039,13 @@
         <v>41</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>49</v>
@@ -1976,23 +2054,26 @@
         <v>51</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+      <c r="N9" s="10" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="25" t="n">
+      <c r="B10" s="26" t="n">
         <f aca="false">IF(A10&gt;Budget!$B$7,"",Budget!$B$5+(A10-1)*7)</f>
         <v>46300</v>
       </c>
@@ -2003,20 +2084,21 @@
       <c r="G10" s="12"/>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
-      <c r="J10" s="13" t="str">
-        <f aca="false">IF(COUNT(C10:I10)=0,"",SUM(C10:I10))</f>
-        <v/>
-      </c>
-      <c r="K10" s="13" t="n">
-        <f aca="false">IF(B10="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L10" s="13" t="str">
-        <f aca="false">IF(J10="","",K10-J10)</f>
-        <v/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="13" t="str">
+        <f aca="false">IF(COUNT(C10:J10)=0,"",SUM(C10:J10))</f>
+        <v/>
+      </c>
+      <c r="L10" s="13" t="n">
+        <f aca="false">IF(B10="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M10" s="13" t="str">
-        <f aca="false">IF(L10="","",SUM($L$10:L10))</f>
+        <f aca="false">IF(K10="","",L10-K10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="13" t="str">
+        <f aca="false">IF(M10="","",SUM($M$10:M10))</f>
         <v/>
       </c>
     </row>
@@ -2024,7 +2106,7 @@
       <c r="A11" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="25" t="n">
+      <c r="B11" s="26" t="n">
         <f aca="false">IF(A11&gt;Budget!$B$7,"",Budget!$B$5+(A11-1)*7)</f>
         <v>46307</v>
       </c>
@@ -2035,20 +2117,21 @@
       <c r="G11" s="12"/>
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
-      <c r="J11" s="13" t="str">
-        <f aca="false">IF(COUNT(C11:I11)=0,"",SUM(C11:I11))</f>
-        <v/>
-      </c>
-      <c r="K11" s="13" t="n">
-        <f aca="false">IF(B11="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L11" s="13" t="str">
-        <f aca="false">IF(J11="","",K11-J11)</f>
-        <v/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="13" t="str">
+        <f aca="false">IF(COUNT(C11:J11)=0,"",SUM(C11:J11))</f>
+        <v/>
+      </c>
+      <c r="L11" s="13" t="n">
+        <f aca="false">IF(B11="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M11" s="13" t="str">
-        <f aca="false">IF(L11="","",SUM($L$10:L11))</f>
+        <f aca="false">IF(K11="","",L11-K11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="13" t="str">
+        <f aca="false">IF(M11="","",SUM($M$10:M11))</f>
         <v/>
       </c>
     </row>
@@ -2056,7 +2139,7 @@
       <c r="A12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="26" t="n">
         <f aca="false">IF(A12&gt;Budget!$B$7,"",Budget!$B$5+(A12-1)*7)</f>
         <v>46314</v>
       </c>
@@ -2067,20 +2150,21 @@
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
-      <c r="J12" s="13" t="str">
-        <f aca="false">IF(COUNT(C12:I12)=0,"",SUM(C12:I12))</f>
-        <v/>
-      </c>
-      <c r="K12" s="13" t="n">
-        <f aca="false">IF(B12="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L12" s="13" t="str">
-        <f aca="false">IF(J12="","",K12-J12)</f>
-        <v/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="13" t="str">
+        <f aca="false">IF(COUNT(C12:J12)=0,"",SUM(C12:J12))</f>
+        <v/>
+      </c>
+      <c r="L12" s="13" t="n">
+        <f aca="false">IF(B12="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M12" s="13" t="str">
-        <f aca="false">IF(L12="","",SUM($L$10:L12))</f>
+        <f aca="false">IF(K12="","",L12-K12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="13" t="str">
+        <f aca="false">IF(M12="","",SUM($M$10:M12))</f>
         <v/>
       </c>
     </row>
@@ -2088,7 +2172,7 @@
       <c r="A13" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B13" s="25" t="n">
+      <c r="B13" s="26" t="n">
         <f aca="false">IF(A13&gt;Budget!$B$7,"",Budget!$B$5+(A13-1)*7)</f>
         <v>46321</v>
       </c>
@@ -2099,20 +2183,21 @@
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
-      <c r="J13" s="13" t="str">
-        <f aca="false">IF(COUNT(C13:I13)=0,"",SUM(C13:I13))</f>
-        <v/>
-      </c>
-      <c r="K13" s="13" t="n">
-        <f aca="false">IF(B13="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L13" s="13" t="str">
-        <f aca="false">IF(J13="","",K13-J13)</f>
-        <v/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="13" t="str">
+        <f aca="false">IF(COUNT(C13:J13)=0,"",SUM(C13:J13))</f>
+        <v/>
+      </c>
+      <c r="L13" s="13" t="n">
+        <f aca="false">IF(B13="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M13" s="13" t="str">
-        <f aca="false">IF(L13="","",SUM($L$10:L13))</f>
+        <f aca="false">IF(K13="","",L13-K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="13" t="str">
+        <f aca="false">IF(M13="","",SUM($M$10:M13))</f>
         <v/>
       </c>
     </row>
@@ -2120,7 +2205,7 @@
       <c r="A14" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B14" s="25" t="n">
+      <c r="B14" s="26" t="n">
         <f aca="false">IF(A14&gt;Budget!$B$7,"",Budget!$B$5+(A14-1)*7)</f>
         <v>46328</v>
       </c>
@@ -2131,20 +2216,21 @@
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
-      <c r="J14" s="13" t="str">
-        <f aca="false">IF(COUNT(C14:I14)=0,"",SUM(C14:I14))</f>
-        <v/>
-      </c>
-      <c r="K14" s="13" t="n">
-        <f aca="false">IF(B14="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L14" s="13" t="str">
-        <f aca="false">IF(J14="","",K14-J14)</f>
-        <v/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="13" t="str">
+        <f aca="false">IF(COUNT(C14:J14)=0,"",SUM(C14:J14))</f>
+        <v/>
+      </c>
+      <c r="L14" s="13" t="n">
+        <f aca="false">IF(B14="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M14" s="13" t="str">
-        <f aca="false">IF(L14="","",SUM($L$10:L14))</f>
+        <f aca="false">IF(K14="","",L14-K14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="13" t="str">
+        <f aca="false">IF(M14="","",SUM($M$10:M14))</f>
         <v/>
       </c>
     </row>
@@ -2152,7 +2238,7 @@
       <c r="A15" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="25" t="n">
+      <c r="B15" s="26" t="n">
         <f aca="false">IF(A15&gt;Budget!$B$7,"",Budget!$B$5+(A15-1)*7)</f>
         <v>46335</v>
       </c>
@@ -2163,20 +2249,21 @@
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
       <c r="I15" s="12"/>
-      <c r="J15" s="13" t="str">
-        <f aca="false">IF(COUNT(C15:I15)=0,"",SUM(C15:I15))</f>
-        <v/>
-      </c>
-      <c r="K15" s="13" t="n">
-        <f aca="false">IF(B15="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L15" s="13" t="str">
-        <f aca="false">IF(J15="","",K15-J15)</f>
-        <v/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="13" t="str">
+        <f aca="false">IF(COUNT(C15:J15)=0,"",SUM(C15:J15))</f>
+        <v/>
+      </c>
+      <c r="L15" s="13" t="n">
+        <f aca="false">IF(B15="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M15" s="13" t="str">
-        <f aca="false">IF(L15="","",SUM($L$10:L15))</f>
+        <f aca="false">IF(K15="","",L15-K15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="13" t="str">
+        <f aca="false">IF(M15="","",SUM($M$10:M15))</f>
         <v/>
       </c>
     </row>
@@ -2184,7 +2271,7 @@
       <c r="A16" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B16" s="25" t="n">
+      <c r="B16" s="26" t="n">
         <f aca="false">IF(A16&gt;Budget!$B$7,"",Budget!$B$5+(A16-1)*7)</f>
         <v>46342</v>
       </c>
@@ -2195,20 +2282,21 @@
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
-      <c r="J16" s="13" t="str">
-        <f aca="false">IF(COUNT(C16:I16)=0,"",SUM(C16:I16))</f>
-        <v/>
-      </c>
-      <c r="K16" s="13" t="n">
-        <f aca="false">IF(B16="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L16" s="13" t="str">
-        <f aca="false">IF(J16="","",K16-J16)</f>
-        <v/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="13" t="str">
+        <f aca="false">IF(COUNT(C16:J16)=0,"",SUM(C16:J16))</f>
+        <v/>
+      </c>
+      <c r="L16" s="13" t="n">
+        <f aca="false">IF(B16="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M16" s="13" t="str">
-        <f aca="false">IF(L16="","",SUM($L$10:L16))</f>
+        <f aca="false">IF(K16="","",L16-K16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="13" t="str">
+        <f aca="false">IF(M16="","",SUM($M$10:M16))</f>
         <v/>
       </c>
     </row>
@@ -2216,7 +2304,7 @@
       <c r="A17" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B17" s="25" t="n">
+      <c r="B17" s="26" t="n">
         <f aca="false">IF(A17&gt;Budget!$B$7,"",Budget!$B$5+(A17-1)*7)</f>
         <v>46349</v>
       </c>
@@ -2227,20 +2315,21 @@
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="13" t="str">
-        <f aca="false">IF(COUNT(C17:I17)=0,"",SUM(C17:I17))</f>
-        <v/>
-      </c>
-      <c r="K17" s="13" t="n">
-        <f aca="false">IF(B17="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L17" s="13" t="str">
-        <f aca="false">IF(J17="","",K17-J17)</f>
-        <v/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="13" t="str">
+        <f aca="false">IF(COUNT(C17:J17)=0,"",SUM(C17:J17))</f>
+        <v/>
+      </c>
+      <c r="L17" s="13" t="n">
+        <f aca="false">IF(B17="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M17" s="13" t="str">
-        <f aca="false">IF(L17="","",SUM($L$10:L17))</f>
+        <f aca="false">IF(K17="","",L17-K17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="13" t="str">
+        <f aca="false">IF(M17="","",SUM($M$10:M17))</f>
         <v/>
       </c>
     </row>
@@ -2248,7 +2337,7 @@
       <c r="A18" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B18" s="25" t="n">
+      <c r="B18" s="26" t="n">
         <f aca="false">IF(A18&gt;Budget!$B$7,"",Budget!$B$5+(A18-1)*7)</f>
         <v>46356</v>
       </c>
@@ -2259,20 +2348,21 @@
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="13" t="str">
-        <f aca="false">IF(COUNT(C18:I18)=0,"",SUM(C18:I18))</f>
-        <v/>
-      </c>
-      <c r="K18" s="13" t="n">
-        <f aca="false">IF(B18="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L18" s="13" t="str">
-        <f aca="false">IF(J18="","",K18-J18)</f>
-        <v/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="13" t="str">
+        <f aca="false">IF(COUNT(C18:J18)=0,"",SUM(C18:J18))</f>
+        <v/>
+      </c>
+      <c r="L18" s="13" t="n">
+        <f aca="false">IF(B18="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M18" s="13" t="str">
-        <f aca="false">IF(L18="","",SUM($L$10:L18))</f>
+        <f aca="false">IF(K18="","",L18-K18)</f>
+        <v/>
+      </c>
+      <c r="N18" s="13" t="str">
+        <f aca="false">IF(M18="","",SUM($M$10:M18))</f>
         <v/>
       </c>
     </row>
@@ -2280,7 +2370,7 @@
       <c r="A19" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B19" s="25" t="n">
+      <c r="B19" s="26" t="n">
         <f aca="false">IF(A19&gt;Budget!$B$7,"",Budget!$B$5+(A19-1)*7)</f>
         <v>46363</v>
       </c>
@@ -2291,20 +2381,21 @@
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
-      <c r="J19" s="13" t="str">
-        <f aca="false">IF(COUNT(C19:I19)=0,"",SUM(C19:I19))</f>
-        <v/>
-      </c>
-      <c r="K19" s="13" t="n">
-        <f aca="false">IF(B19="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L19" s="13" t="str">
-        <f aca="false">IF(J19="","",K19-J19)</f>
-        <v/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="13" t="str">
+        <f aca="false">IF(COUNT(C19:J19)=0,"",SUM(C19:J19))</f>
+        <v/>
+      </c>
+      <c r="L19" s="13" t="n">
+        <f aca="false">IF(B19="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M19" s="13" t="str">
-        <f aca="false">IF(L19="","",SUM($L$10:L19))</f>
+        <f aca="false">IF(K19="","",L19-K19)</f>
+        <v/>
+      </c>
+      <c r="N19" s="13" t="str">
+        <f aca="false">IF(M19="","",SUM($M$10:M19))</f>
         <v/>
       </c>
     </row>
@@ -2312,7 +2403,7 @@
       <c r="A20" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="25" t="n">
+      <c r="B20" s="26" t="n">
         <f aca="false">IF(A20&gt;Budget!$B$7,"",Budget!$B$5+(A20-1)*7)</f>
         <v>46370</v>
       </c>
@@ -2323,20 +2414,21 @@
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>
-      <c r="J20" s="13" t="str">
-        <f aca="false">IF(COUNT(C20:I20)=0,"",SUM(C20:I20))</f>
-        <v/>
-      </c>
-      <c r="K20" s="13" t="n">
-        <f aca="false">IF(B20="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L20" s="13" t="str">
-        <f aca="false">IF(J20="","",K20-J20)</f>
-        <v/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="13" t="str">
+        <f aca="false">IF(COUNT(C20:J20)=0,"",SUM(C20:J20))</f>
+        <v/>
+      </c>
+      <c r="L20" s="13" t="n">
+        <f aca="false">IF(B20="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M20" s="13" t="str">
-        <f aca="false">IF(L20="","",SUM($L$10:L20))</f>
+        <f aca="false">IF(K20="","",L20-K20)</f>
+        <v/>
+      </c>
+      <c r="N20" s="13" t="str">
+        <f aca="false">IF(M20="","",SUM($M$10:M20))</f>
         <v/>
       </c>
     </row>
@@ -2344,7 +2436,7 @@
       <c r="A21" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B21" s="25" t="n">
+      <c r="B21" s="26" t="n">
         <f aca="false">IF(A21&gt;Budget!$B$7,"",Budget!$B$5+(A21-1)*7)</f>
         <v>46377</v>
       </c>
@@ -2355,20 +2447,21 @@
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
-      <c r="J21" s="13" t="str">
-        <f aca="false">IF(COUNT(C21:I21)=0,"",SUM(C21:I21))</f>
-        <v/>
-      </c>
-      <c r="K21" s="13" t="n">
-        <f aca="false">IF(B21="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L21" s="13" t="str">
-        <f aca="false">IF(J21="","",K21-J21)</f>
-        <v/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="13" t="str">
+        <f aca="false">IF(COUNT(C21:J21)=0,"",SUM(C21:J21))</f>
+        <v/>
+      </c>
+      <c r="L21" s="13" t="n">
+        <f aca="false">IF(B21="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M21" s="13" t="str">
-        <f aca="false">IF(L21="","",SUM($L$10:L21))</f>
+        <f aca="false">IF(K21="","",L21-K21)</f>
+        <v/>
+      </c>
+      <c r="N21" s="13" t="str">
+        <f aca="false">IF(M21="","",SUM($M$10:M21))</f>
         <v/>
       </c>
     </row>
@@ -2376,7 +2469,7 @@
       <c r="A22" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B22" s="25" t="n">
+      <c r="B22" s="26" t="n">
         <f aca="false">IF(A22&gt;Budget!$B$7,"",Budget!$B$5+(A22-1)*7)</f>
         <v>46384</v>
       </c>
@@ -2387,20 +2480,21 @@
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
       <c r="I22" s="12"/>
-      <c r="J22" s="13" t="str">
-        <f aca="false">IF(COUNT(C22:I22)=0,"",SUM(C22:I22))</f>
-        <v/>
-      </c>
-      <c r="K22" s="13" t="n">
-        <f aca="false">IF(B22="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L22" s="13" t="str">
-        <f aca="false">IF(J22="","",K22-J22)</f>
-        <v/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="13" t="str">
+        <f aca="false">IF(COUNT(C22:J22)=0,"",SUM(C22:J22))</f>
+        <v/>
+      </c>
+      <c r="L22" s="13" t="n">
+        <f aca="false">IF(B22="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M22" s="13" t="str">
-        <f aca="false">IF(L22="","",SUM($L$10:L22))</f>
+        <f aca="false">IF(K22="","",L22-K22)</f>
+        <v/>
+      </c>
+      <c r="N22" s="13" t="str">
+        <f aca="false">IF(M22="","",SUM($M$10:M22))</f>
         <v/>
       </c>
     </row>
@@ -2408,7 +2502,7 @@
       <c r="A23" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B23" s="25" t="n">
+      <c r="B23" s="26" t="n">
         <f aca="false">IF(A23&gt;Budget!$B$7,"",Budget!$B$5+(A23-1)*7)</f>
         <v>46391</v>
       </c>
@@ -2419,20 +2513,21 @@
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
       <c r="I23" s="12"/>
-      <c r="J23" s="13" t="str">
-        <f aca="false">IF(COUNT(C23:I23)=0,"",SUM(C23:I23))</f>
-        <v/>
-      </c>
-      <c r="K23" s="13" t="n">
-        <f aca="false">IF(B23="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L23" s="13" t="str">
-        <f aca="false">IF(J23="","",K23-J23)</f>
-        <v/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="13" t="str">
+        <f aca="false">IF(COUNT(C23:J23)=0,"",SUM(C23:J23))</f>
+        <v/>
+      </c>
+      <c r="L23" s="13" t="n">
+        <f aca="false">IF(B23="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M23" s="13" t="str">
-        <f aca="false">IF(L23="","",SUM($L$10:L23))</f>
+        <f aca="false">IF(K23="","",L23-K23)</f>
+        <v/>
+      </c>
+      <c r="N23" s="13" t="str">
+        <f aca="false">IF(M23="","",SUM($M$10:M23))</f>
         <v/>
       </c>
     </row>
@@ -2440,7 +2535,7 @@
       <c r="A24" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B24" s="25" t="n">
+      <c r="B24" s="26" t="n">
         <f aca="false">IF(A24&gt;Budget!$B$7,"",Budget!$B$5+(A24-1)*7)</f>
         <v>46398</v>
       </c>
@@ -2451,20 +2546,21 @@
       <c r="G24" s="12"/>
       <c r="H24" s="12"/>
       <c r="I24" s="12"/>
-      <c r="J24" s="13" t="str">
-        <f aca="false">IF(COUNT(C24:I24)=0,"",SUM(C24:I24))</f>
-        <v/>
-      </c>
-      <c r="K24" s="13" t="n">
-        <f aca="false">IF(B24="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L24" s="13" t="str">
-        <f aca="false">IF(J24="","",K24-J24)</f>
-        <v/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="13" t="str">
+        <f aca="false">IF(COUNT(C24:J24)=0,"",SUM(C24:J24))</f>
+        <v/>
+      </c>
+      <c r="L24" s="13" t="n">
+        <f aca="false">IF(B24="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M24" s="13" t="str">
-        <f aca="false">IF(L24="","",SUM($L$10:L24))</f>
+        <f aca="false">IF(K24="","",L24-K24)</f>
+        <v/>
+      </c>
+      <c r="N24" s="13" t="str">
+        <f aca="false">IF(M24="","",SUM($M$10:M24))</f>
         <v/>
       </c>
     </row>
@@ -2472,7 +2568,7 @@
       <c r="A25" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B25" s="25" t="n">
+      <c r="B25" s="26" t="n">
         <f aca="false">IF(A25&gt;Budget!$B$7,"",Budget!$B$5+(A25-1)*7)</f>
         <v>46405</v>
       </c>
@@ -2483,20 +2579,21 @@
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
-      <c r="J25" s="13" t="str">
-        <f aca="false">IF(COUNT(C25:I25)=0,"",SUM(C25:I25))</f>
-        <v/>
-      </c>
-      <c r="K25" s="13" t="n">
-        <f aca="false">IF(B25="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L25" s="13" t="str">
-        <f aca="false">IF(J25="","",K25-J25)</f>
-        <v/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="13" t="str">
+        <f aca="false">IF(COUNT(C25:J25)=0,"",SUM(C25:J25))</f>
+        <v/>
+      </c>
+      <c r="L25" s="13" t="n">
+        <f aca="false">IF(B25="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M25" s="13" t="str">
-        <f aca="false">IF(L25="","",SUM($L$10:L25))</f>
+        <f aca="false">IF(K25="","",L25-K25)</f>
+        <v/>
+      </c>
+      <c r="N25" s="13" t="str">
+        <f aca="false">IF(M25="","",SUM($M$10:M25))</f>
         <v/>
       </c>
     </row>
@@ -2504,7 +2601,7 @@
       <c r="A26" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B26" s="25" t="n">
+      <c r="B26" s="26" t="n">
         <f aca="false">IF(A26&gt;Budget!$B$7,"",Budget!$B$5+(A26-1)*7)</f>
         <v>46412</v>
       </c>
@@ -2515,20 +2612,21 @@
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
       <c r="I26" s="12"/>
-      <c r="J26" s="13" t="str">
-        <f aca="false">IF(COUNT(C26:I26)=0,"",SUM(C26:I26))</f>
-        <v/>
-      </c>
-      <c r="K26" s="13" t="n">
-        <f aca="false">IF(B26="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L26" s="13" t="str">
-        <f aca="false">IF(J26="","",K26-J26)</f>
-        <v/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="13" t="str">
+        <f aca="false">IF(COUNT(C26:J26)=0,"",SUM(C26:J26))</f>
+        <v/>
+      </c>
+      <c r="L26" s="13" t="n">
+        <f aca="false">IF(B26="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M26" s="13" t="str">
-        <f aca="false">IF(L26="","",SUM($L$10:L26))</f>
+        <f aca="false">IF(K26="","",L26-K26)</f>
+        <v/>
+      </c>
+      <c r="N26" s="13" t="str">
+        <f aca="false">IF(M26="","",SUM($M$10:M26))</f>
         <v/>
       </c>
     </row>
@@ -2536,7 +2634,7 @@
       <c r="A27" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B27" s="25" t="n">
+      <c r="B27" s="26" t="n">
         <f aca="false">IF(A27&gt;Budget!$B$7,"",Budget!$B$5+(A27-1)*7)</f>
         <v>46419</v>
       </c>
@@ -2547,20 +2645,21 @@
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
       <c r="I27" s="12"/>
-      <c r="J27" s="13" t="str">
-        <f aca="false">IF(COUNT(C27:I27)=0,"",SUM(C27:I27))</f>
-        <v/>
-      </c>
-      <c r="K27" s="13" t="n">
-        <f aca="false">IF(B27="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L27" s="13" t="str">
-        <f aca="false">IF(J27="","",K27-J27)</f>
-        <v/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="13" t="str">
+        <f aca="false">IF(COUNT(C27:J27)=0,"",SUM(C27:J27))</f>
+        <v/>
+      </c>
+      <c r="L27" s="13" t="n">
+        <f aca="false">IF(B27="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M27" s="13" t="str">
-        <f aca="false">IF(L27="","",SUM($L$10:L27))</f>
+        <f aca="false">IF(K27="","",L27-K27)</f>
+        <v/>
+      </c>
+      <c r="N27" s="13" t="str">
+        <f aca="false">IF(M27="","",SUM($M$10:M27))</f>
         <v/>
       </c>
     </row>
@@ -2568,7 +2667,7 @@
       <c r="A28" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B28" s="25" t="n">
+      <c r="B28" s="26" t="n">
         <f aca="false">IF(A28&gt;Budget!$B$7,"",Budget!$B$5+(A28-1)*7)</f>
         <v>46426</v>
       </c>
@@ -2579,20 +2678,21 @@
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
       <c r="I28" s="12"/>
-      <c r="J28" s="13" t="str">
-        <f aca="false">IF(COUNT(C28:I28)=0,"",SUM(C28:I28))</f>
-        <v/>
-      </c>
-      <c r="K28" s="13" t="n">
-        <f aca="false">IF(B28="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L28" s="13" t="str">
-        <f aca="false">IF(J28="","",K28-J28)</f>
-        <v/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="13" t="str">
+        <f aca="false">IF(COUNT(C28:J28)=0,"",SUM(C28:J28))</f>
+        <v/>
+      </c>
+      <c r="L28" s="13" t="n">
+        <f aca="false">IF(B28="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M28" s="13" t="str">
-        <f aca="false">IF(L28="","",SUM($L$10:L28))</f>
+        <f aca="false">IF(K28="","",L28-K28)</f>
+        <v/>
+      </c>
+      <c r="N28" s="13" t="str">
+        <f aca="false">IF(M28="","",SUM($M$10:M28))</f>
         <v/>
       </c>
     </row>
@@ -2600,7 +2700,7 @@
       <c r="A29" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B29" s="25" t="n">
+      <c r="B29" s="26" t="n">
         <f aca="false">IF(A29&gt;Budget!$B$7,"",Budget!$B$5+(A29-1)*7)</f>
         <v>46433</v>
       </c>
@@ -2611,20 +2711,21 @@
       <c r="G29" s="12"/>
       <c r="H29" s="12"/>
       <c r="I29" s="12"/>
-      <c r="J29" s="13" t="str">
-        <f aca="false">IF(COUNT(C29:I29)=0,"",SUM(C29:I29))</f>
-        <v/>
-      </c>
-      <c r="K29" s="13" t="n">
-        <f aca="false">IF(B29="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L29" s="13" t="str">
-        <f aca="false">IF(J29="","",K29-J29)</f>
-        <v/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="13" t="str">
+        <f aca="false">IF(COUNT(C29:J29)=0,"",SUM(C29:J29))</f>
+        <v/>
+      </c>
+      <c r="L29" s="13" t="n">
+        <f aca="false">IF(B29="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M29" s="13" t="str">
-        <f aca="false">IF(L29="","",SUM($L$10:L29))</f>
+        <f aca="false">IF(K29="","",L29-K29)</f>
+        <v/>
+      </c>
+      <c r="N29" s="13" t="str">
+        <f aca="false">IF(M29="","",SUM($M$10:M29))</f>
         <v/>
       </c>
     </row>
@@ -2632,7 +2733,7 @@
       <c r="A30" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B30" s="25" t="n">
+      <c r="B30" s="26" t="n">
         <f aca="false">IF(A30&gt;Budget!$B$7,"",Budget!$B$5+(A30-1)*7)</f>
         <v>46440</v>
       </c>
@@ -2643,20 +2744,21 @@
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="13" t="str">
-        <f aca="false">IF(COUNT(C30:I30)=0,"",SUM(C30:I30))</f>
-        <v/>
-      </c>
-      <c r="K30" s="13" t="n">
-        <f aca="false">IF(B30="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L30" s="13" t="str">
-        <f aca="false">IF(J30="","",K30-J30)</f>
-        <v/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="13" t="str">
+        <f aca="false">IF(COUNT(C30:J30)=0,"",SUM(C30:J30))</f>
+        <v/>
+      </c>
+      <c r="L30" s="13" t="n">
+        <f aca="false">IF(B30="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M30" s="13" t="str">
-        <f aca="false">IF(L30="","",SUM($L$10:L30))</f>
+        <f aca="false">IF(K30="","",L30-K30)</f>
+        <v/>
+      </c>
+      <c r="N30" s="13" t="str">
+        <f aca="false">IF(M30="","",SUM($M$10:M30))</f>
         <v/>
       </c>
     </row>
@@ -2664,7 +2766,7 @@
       <c r="A31" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B31" s="25" t="n">
+      <c r="B31" s="26" t="n">
         <f aca="false">IF(A31&gt;Budget!$B$7,"",Budget!$B$5+(A31-1)*7)</f>
         <v>46447</v>
       </c>
@@ -2675,20 +2777,21 @@
       <c r="G31" s="12"/>
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
-      <c r="J31" s="13" t="str">
-        <f aca="false">IF(COUNT(C31:I31)=0,"",SUM(C31:I31))</f>
-        <v/>
-      </c>
-      <c r="K31" s="13" t="n">
-        <f aca="false">IF(B31="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L31" s="13" t="str">
-        <f aca="false">IF(J31="","",K31-J31)</f>
-        <v/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="13" t="str">
+        <f aca="false">IF(COUNT(C31:J31)=0,"",SUM(C31:J31))</f>
+        <v/>
+      </c>
+      <c r="L31" s="13" t="n">
+        <f aca="false">IF(B31="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M31" s="13" t="str">
-        <f aca="false">IF(L31="","",SUM($L$10:L31))</f>
+        <f aca="false">IF(K31="","",L31-K31)</f>
+        <v/>
+      </c>
+      <c r="N31" s="13" t="str">
+        <f aca="false">IF(M31="","",SUM($M$10:M31))</f>
         <v/>
       </c>
     </row>
@@ -2696,7 +2799,7 @@
       <c r="A32" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B32" s="25" t="n">
+      <c r="B32" s="26" t="n">
         <f aca="false">IF(A32&gt;Budget!$B$7,"",Budget!$B$5+(A32-1)*7)</f>
         <v>46454</v>
       </c>
@@ -2707,20 +2810,21 @@
       <c r="G32" s="12"/>
       <c r="H32" s="12"/>
       <c r="I32" s="12"/>
-      <c r="J32" s="13" t="str">
-        <f aca="false">IF(COUNT(C32:I32)=0,"",SUM(C32:I32))</f>
-        <v/>
-      </c>
-      <c r="K32" s="13" t="n">
-        <f aca="false">IF(B32="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L32" s="13" t="str">
-        <f aca="false">IF(J32="","",K32-J32)</f>
-        <v/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="13" t="str">
+        <f aca="false">IF(COUNT(C32:J32)=0,"",SUM(C32:J32))</f>
+        <v/>
+      </c>
+      <c r="L32" s="13" t="n">
+        <f aca="false">IF(B32="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M32" s="13" t="str">
-        <f aca="false">IF(L32="","",SUM($L$10:L32))</f>
+        <f aca="false">IF(K32="","",L32-K32)</f>
+        <v/>
+      </c>
+      <c r="N32" s="13" t="str">
+        <f aca="false">IF(M32="","",SUM($M$10:M32))</f>
         <v/>
       </c>
     </row>
@@ -2728,7 +2832,7 @@
       <c r="A33" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B33" s="25" t="n">
+      <c r="B33" s="26" t="n">
         <f aca="false">IF(A33&gt;Budget!$B$7,"",Budget!$B$5+(A33-1)*7)</f>
         <v>46461</v>
       </c>
@@ -2739,20 +2843,21 @@
       <c r="G33" s="12"/>
       <c r="H33" s="12"/>
       <c r="I33" s="12"/>
-      <c r="J33" s="13" t="str">
-        <f aca="false">IF(COUNT(C33:I33)=0,"",SUM(C33:I33))</f>
-        <v/>
-      </c>
-      <c r="K33" s="13" t="n">
-        <f aca="false">IF(B33="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L33" s="13" t="str">
-        <f aca="false">IF(J33="","",K33-J33)</f>
-        <v/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="13" t="str">
+        <f aca="false">IF(COUNT(C33:J33)=0,"",SUM(C33:J33))</f>
+        <v/>
+      </c>
+      <c r="L33" s="13" t="n">
+        <f aca="false">IF(B33="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M33" s="13" t="str">
-        <f aca="false">IF(L33="","",SUM($L$10:L33))</f>
+        <f aca="false">IF(K33="","",L33-K33)</f>
+        <v/>
+      </c>
+      <c r="N33" s="13" t="str">
+        <f aca="false">IF(M33="","",SUM($M$10:M33))</f>
         <v/>
       </c>
     </row>
@@ -2760,7 +2865,7 @@
       <c r="A34" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="B34" s="25" t="n">
+      <c r="B34" s="26" t="n">
         <f aca="false">IF(A34&gt;Budget!$B$7,"",Budget!$B$5+(A34-1)*7)</f>
         <v>46468</v>
       </c>
@@ -2771,20 +2876,21 @@
       <c r="G34" s="12"/>
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
-      <c r="J34" s="13" t="str">
-        <f aca="false">IF(COUNT(C34:I34)=0,"",SUM(C34:I34))</f>
-        <v/>
-      </c>
-      <c r="K34" s="13" t="n">
-        <f aca="false">IF(B34="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L34" s="13" t="str">
-        <f aca="false">IF(J34="","",K34-J34)</f>
-        <v/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="13" t="str">
+        <f aca="false">IF(COUNT(C34:J34)=0,"",SUM(C34:J34))</f>
+        <v/>
+      </c>
+      <c r="L34" s="13" t="n">
+        <f aca="false">IF(B34="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M34" s="13" t="str">
-        <f aca="false">IF(L34="","",SUM($L$10:L34))</f>
+        <f aca="false">IF(K34="","",L34-K34)</f>
+        <v/>
+      </c>
+      <c r="N34" s="13" t="str">
+        <f aca="false">IF(M34="","",SUM($M$10:M34))</f>
         <v/>
       </c>
     </row>
@@ -2792,7 +2898,7 @@
       <c r="A35" s="11" t="n">
         <v>26</v>
       </c>
-      <c r="B35" s="25" t="n">
+      <c r="B35" s="26" t="n">
         <f aca="false">IF(A35&gt;Budget!$B$7,"",Budget!$B$5+(A35-1)*7)</f>
         <v>46475</v>
       </c>
@@ -2803,20 +2909,21 @@
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
       <c r="I35" s="12"/>
-      <c r="J35" s="13" t="str">
-        <f aca="false">IF(COUNT(C35:I35)=0,"",SUM(C35:I35))</f>
-        <v/>
-      </c>
-      <c r="K35" s="13" t="n">
-        <f aca="false">IF(B35="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L35" s="13" t="str">
-        <f aca="false">IF(J35="","",K35-J35)</f>
-        <v/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="13" t="str">
+        <f aca="false">IF(COUNT(C35:J35)=0,"",SUM(C35:J35))</f>
+        <v/>
+      </c>
+      <c r="L35" s="13" t="n">
+        <f aca="false">IF(B35="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M35" s="13" t="str">
-        <f aca="false">IF(L35="","",SUM($L$10:L35))</f>
+        <f aca="false">IF(K35="","",L35-K35)</f>
+        <v/>
+      </c>
+      <c r="N35" s="13" t="str">
+        <f aca="false">IF(M35="","",SUM($M$10:M35))</f>
         <v/>
       </c>
     </row>
@@ -2824,7 +2931,7 @@
       <c r="A36" s="11" t="n">
         <v>27</v>
       </c>
-      <c r="B36" s="25" t="n">
+      <c r="B36" s="26" t="n">
         <f aca="false">IF(A36&gt;Budget!$B$7,"",Budget!$B$5+(A36-1)*7)</f>
         <v>46482</v>
       </c>
@@ -2835,20 +2942,21 @@
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
-      <c r="J36" s="13" t="str">
-        <f aca="false">IF(COUNT(C36:I36)=0,"",SUM(C36:I36))</f>
-        <v/>
-      </c>
-      <c r="K36" s="13" t="n">
-        <f aca="false">IF(B36="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L36" s="13" t="str">
-        <f aca="false">IF(J36="","",K36-J36)</f>
-        <v/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="13" t="str">
+        <f aca="false">IF(COUNT(C36:J36)=0,"",SUM(C36:J36))</f>
+        <v/>
+      </c>
+      <c r="L36" s="13" t="n">
+        <f aca="false">IF(B36="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M36" s="13" t="str">
-        <f aca="false">IF(L36="","",SUM($L$10:L36))</f>
+        <f aca="false">IF(K36="","",L36-K36)</f>
+        <v/>
+      </c>
+      <c r="N36" s="13" t="str">
+        <f aca="false">IF(M36="","",SUM($M$10:M36))</f>
         <v/>
       </c>
     </row>
@@ -2856,7 +2964,7 @@
       <c r="A37" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="B37" s="25" t="n">
+      <c r="B37" s="26" t="n">
         <f aca="false">IF(A37&gt;Budget!$B$7,"",Budget!$B$5+(A37-1)*7)</f>
         <v>46489</v>
       </c>
@@ -2867,20 +2975,21 @@
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
       <c r="I37" s="12"/>
-      <c r="J37" s="13" t="str">
-        <f aca="false">IF(COUNT(C37:I37)=0,"",SUM(C37:I37))</f>
-        <v/>
-      </c>
-      <c r="K37" s="13" t="n">
-        <f aca="false">IF(B37="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L37" s="13" t="str">
-        <f aca="false">IF(J37="","",K37-J37)</f>
-        <v/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="13" t="str">
+        <f aca="false">IF(COUNT(C37:J37)=0,"",SUM(C37:J37))</f>
+        <v/>
+      </c>
+      <c r="L37" s="13" t="n">
+        <f aca="false">IF(B37="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M37" s="13" t="str">
-        <f aca="false">IF(L37="","",SUM($L$10:L37))</f>
+        <f aca="false">IF(K37="","",L37-K37)</f>
+        <v/>
+      </c>
+      <c r="N37" s="13" t="str">
+        <f aca="false">IF(M37="","",SUM($M$10:M37))</f>
         <v/>
       </c>
     </row>
@@ -2888,7 +2997,7 @@
       <c r="A38" s="11" t="n">
         <v>29</v>
       </c>
-      <c r="B38" s="25" t="n">
+      <c r="B38" s="26" t="n">
         <f aca="false">IF(A38&gt;Budget!$B$7,"",Budget!$B$5+(A38-1)*7)</f>
         <v>46496</v>
       </c>
@@ -2899,20 +3008,21 @@
       <c r="G38" s="12"/>
       <c r="H38" s="12"/>
       <c r="I38" s="12"/>
-      <c r="J38" s="13" t="str">
-        <f aca="false">IF(COUNT(C38:I38)=0,"",SUM(C38:I38))</f>
-        <v/>
-      </c>
-      <c r="K38" s="13" t="n">
-        <f aca="false">IF(B38="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L38" s="13" t="str">
-        <f aca="false">IF(J38="","",K38-J38)</f>
-        <v/>
+      <c r="J38" s="12"/>
+      <c r="K38" s="13" t="str">
+        <f aca="false">IF(COUNT(C38:J38)=0,"",SUM(C38:J38))</f>
+        <v/>
+      </c>
+      <c r="L38" s="13" t="n">
+        <f aca="false">IF(B38="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M38" s="13" t="str">
-        <f aca="false">IF(L38="","",SUM($L$10:L38))</f>
+        <f aca="false">IF(K38="","",L38-K38)</f>
+        <v/>
+      </c>
+      <c r="N38" s="13" t="str">
+        <f aca="false">IF(M38="","",SUM($M$10:M38))</f>
         <v/>
       </c>
     </row>
@@ -2920,7 +3030,7 @@
       <c r="A39" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="B39" s="25" t="n">
+      <c r="B39" s="26" t="n">
         <f aca="false">IF(A39&gt;Budget!$B$7,"",Budget!$B$5+(A39-1)*7)</f>
         <v>46503</v>
       </c>
@@ -2931,20 +3041,21 @@
       <c r="G39" s="12"/>
       <c r="H39" s="12"/>
       <c r="I39" s="12"/>
-      <c r="J39" s="13" t="str">
-        <f aca="false">IF(COUNT(C39:I39)=0,"",SUM(C39:I39))</f>
-        <v/>
-      </c>
-      <c r="K39" s="13" t="n">
-        <f aca="false">IF(B39="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L39" s="13" t="str">
-        <f aca="false">IF(J39="","",K39-J39)</f>
-        <v/>
+      <c r="J39" s="12"/>
+      <c r="K39" s="13" t="str">
+        <f aca="false">IF(COUNT(C39:J39)=0,"",SUM(C39:J39))</f>
+        <v/>
+      </c>
+      <c r="L39" s="13" t="n">
+        <f aca="false">IF(B39="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M39" s="13" t="str">
-        <f aca="false">IF(L39="","",SUM($L$10:L39))</f>
+        <f aca="false">IF(K39="","",L39-K39)</f>
+        <v/>
+      </c>
+      <c r="N39" s="13" t="str">
+        <f aca="false">IF(M39="","",SUM($M$10:M39))</f>
         <v/>
       </c>
     </row>
@@ -2952,7 +3063,7 @@
       <c r="A40" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="B40" s="25" t="n">
+      <c r="B40" s="26" t="n">
         <f aca="false">IF(A40&gt;Budget!$B$7,"",Budget!$B$5+(A40-1)*7)</f>
         <v>46510</v>
       </c>
@@ -2963,20 +3074,21 @@
       <c r="G40" s="12"/>
       <c r="H40" s="12"/>
       <c r="I40" s="12"/>
-      <c r="J40" s="13" t="str">
-        <f aca="false">IF(COUNT(C40:I40)=0,"",SUM(C40:I40))</f>
-        <v/>
-      </c>
-      <c r="K40" s="13" t="n">
-        <f aca="false">IF(B40="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L40" s="13" t="str">
-        <f aca="false">IF(J40="","",K40-J40)</f>
-        <v/>
+      <c r="J40" s="12"/>
+      <c r="K40" s="13" t="str">
+        <f aca="false">IF(COUNT(C40:J40)=0,"",SUM(C40:J40))</f>
+        <v/>
+      </c>
+      <c r="L40" s="13" t="n">
+        <f aca="false">IF(B40="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M40" s="13" t="str">
-        <f aca="false">IF(L40="","",SUM($L$10:L40))</f>
+        <f aca="false">IF(K40="","",L40-K40)</f>
+        <v/>
+      </c>
+      <c r="N40" s="13" t="str">
+        <f aca="false">IF(M40="","",SUM($M$10:M40))</f>
         <v/>
       </c>
     </row>
@@ -2984,7 +3096,7 @@
       <c r="A41" s="11" t="n">
         <v>32</v>
       </c>
-      <c r="B41" s="25" t="n">
+      <c r="B41" s="26" t="n">
         <f aca="false">IF(A41&gt;Budget!$B$7,"",Budget!$B$5+(A41-1)*7)</f>
         <v>46517</v>
       </c>
@@ -2995,20 +3107,21 @@
       <c r="G41" s="12"/>
       <c r="H41" s="12"/>
       <c r="I41" s="12"/>
-      <c r="J41" s="13" t="str">
-        <f aca="false">IF(COUNT(C41:I41)=0,"",SUM(C41:I41))</f>
-        <v/>
-      </c>
-      <c r="K41" s="13" t="n">
-        <f aca="false">IF(B41="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L41" s="13" t="str">
-        <f aca="false">IF(J41="","",K41-J41)</f>
-        <v/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="13" t="str">
+        <f aca="false">IF(COUNT(C41:J41)=0,"",SUM(C41:J41))</f>
+        <v/>
+      </c>
+      <c r="L41" s="13" t="n">
+        <f aca="false">IF(B41="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M41" s="13" t="str">
-        <f aca="false">IF(L41="","",SUM($L$10:L41))</f>
+        <f aca="false">IF(K41="","",L41-K41)</f>
+        <v/>
+      </c>
+      <c r="N41" s="13" t="str">
+        <f aca="false">IF(M41="","",SUM($M$10:M41))</f>
         <v/>
       </c>
     </row>
@@ -3016,7 +3129,7 @@
       <c r="A42" s="11" t="n">
         <v>33</v>
       </c>
-      <c r="B42" s="25" t="n">
+      <c r="B42" s="26" t="n">
         <f aca="false">IF(A42&gt;Budget!$B$7,"",Budget!$B$5+(A42-1)*7)</f>
         <v>46524</v>
       </c>
@@ -3027,20 +3140,21 @@
       <c r="G42" s="12"/>
       <c r="H42" s="12"/>
       <c r="I42" s="12"/>
-      <c r="J42" s="13" t="str">
-        <f aca="false">IF(COUNT(C42:I42)=0,"",SUM(C42:I42))</f>
-        <v/>
-      </c>
-      <c r="K42" s="13" t="n">
-        <f aca="false">IF(B42="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L42" s="13" t="str">
-        <f aca="false">IF(J42="","",K42-J42)</f>
-        <v/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="13" t="str">
+        <f aca="false">IF(COUNT(C42:J42)=0,"",SUM(C42:J42))</f>
+        <v/>
+      </c>
+      <c r="L42" s="13" t="n">
+        <f aca="false">IF(B42="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M42" s="13" t="str">
-        <f aca="false">IF(L42="","",SUM($L$10:L42))</f>
+        <f aca="false">IF(K42="","",L42-K42)</f>
+        <v/>
+      </c>
+      <c r="N42" s="13" t="str">
+        <f aca="false">IF(M42="","",SUM($M$10:M42))</f>
         <v/>
       </c>
     </row>
@@ -3048,7 +3162,7 @@
       <c r="A43" s="11" t="n">
         <v>34</v>
       </c>
-      <c r="B43" s="25" t="n">
+      <c r="B43" s="26" t="n">
         <f aca="false">IF(A43&gt;Budget!$B$7,"",Budget!$B$5+(A43-1)*7)</f>
         <v>46531</v>
       </c>
@@ -3059,20 +3173,21 @@
       <c r="G43" s="12"/>
       <c r="H43" s="12"/>
       <c r="I43" s="12"/>
-      <c r="J43" s="13" t="str">
-        <f aca="false">IF(COUNT(C43:I43)=0,"",SUM(C43:I43))</f>
-        <v/>
-      </c>
-      <c r="K43" s="13" t="n">
-        <f aca="false">IF(B43="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L43" s="13" t="str">
-        <f aca="false">IF(J43="","",K43-J43)</f>
-        <v/>
+      <c r="J43" s="12"/>
+      <c r="K43" s="13" t="str">
+        <f aca="false">IF(COUNT(C43:J43)=0,"",SUM(C43:J43))</f>
+        <v/>
+      </c>
+      <c r="L43" s="13" t="n">
+        <f aca="false">IF(B43="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M43" s="13" t="str">
-        <f aca="false">IF(L43="","",SUM($L$10:L43))</f>
+        <f aca="false">IF(K43="","",L43-K43)</f>
+        <v/>
+      </c>
+      <c r="N43" s="13" t="str">
+        <f aca="false">IF(M43="","",SUM($M$10:M43))</f>
         <v/>
       </c>
     </row>
@@ -3080,7 +3195,7 @@
       <c r="A44" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="B44" s="25" t="n">
+      <c r="B44" s="26" t="n">
         <f aca="false">IF(A44&gt;Budget!$B$7,"",Budget!$B$5+(A44-1)*7)</f>
         <v>46538</v>
       </c>
@@ -3091,20 +3206,21 @@
       <c r="G44" s="12"/>
       <c r="H44" s="12"/>
       <c r="I44" s="12"/>
-      <c r="J44" s="13" t="str">
-        <f aca="false">IF(COUNT(C44:I44)=0,"",SUM(C44:I44))</f>
-        <v/>
-      </c>
-      <c r="K44" s="13" t="n">
-        <f aca="false">IF(B44="","",$J$5)</f>
-        <v>128.5</v>
-      </c>
-      <c r="L44" s="13" t="str">
-        <f aca="false">IF(J44="","",K44-J44)</f>
-        <v/>
+      <c r="J44" s="12"/>
+      <c r="K44" s="13" t="str">
+        <f aca="false">IF(COUNT(C44:J44)=0,"",SUM(C44:J44))</f>
+        <v/>
+      </c>
+      <c r="L44" s="13" t="n">
+        <f aca="false">IF(B44="","",$K$5)</f>
+        <v>166.9</v>
       </c>
       <c r="M44" s="13" t="str">
-        <f aca="false">IF(L44="","",SUM($L$10:L44))</f>
+        <f aca="false">IF(K44="","",L44-K44)</f>
+        <v/>
+      </c>
+      <c r="N44" s="13" t="str">
+        <f aca="false">IF(M44="","",SUM($M$10:M44))</f>
         <v/>
       </c>
     </row>
@@ -3112,7 +3228,7 @@
       <c r="A45" s="11" t="n">
         <v>36</v>
       </c>
-      <c r="B45" s="25" t="str">
+      <c r="B45" s="26" t="str">
         <f aca="false">IF(A45&gt;Budget!$B$7,"",Budget!$B$5+(A45-1)*7)</f>
         <v/>
       </c>
@@ -3123,20 +3239,21 @@
       <c r="G45" s="12"/>
       <c r="H45" s="12"/>
       <c r="I45" s="12"/>
-      <c r="J45" s="13" t="str">
-        <f aca="false">IF(COUNT(C45:I45)=0,"",SUM(C45:I45))</f>
-        <v/>
-      </c>
+      <c r="J45" s="12"/>
       <c r="K45" s="13" t="str">
-        <f aca="false">IF(B45="","",$J$5)</f>
+        <f aca="false">IF(COUNT(C45:J45)=0,"",SUM(C45:J45))</f>
         <v/>
       </c>
       <c r="L45" s="13" t="str">
-        <f aca="false">IF(J45="","",K45-J45)</f>
+        <f aca="false">IF(B45="","",$K$5)</f>
         <v/>
       </c>
       <c r="M45" s="13" t="str">
-        <f aca="false">IF(L45="","",SUM($L$10:L45))</f>
+        <f aca="false">IF(K45="","",L45-K45)</f>
+        <v/>
+      </c>
+      <c r="N45" s="13" t="str">
+        <f aca="false">IF(M45="","",SUM($M$10:M45))</f>
         <v/>
       </c>
     </row>
@@ -3144,7 +3261,7 @@
       <c r="A46" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="B46" s="25" t="str">
+      <c r="B46" s="26" t="str">
         <f aca="false">IF(A46&gt;Budget!$B$7,"",Budget!$B$5+(A46-1)*7)</f>
         <v/>
       </c>
@@ -3155,20 +3272,21 @@
       <c r="G46" s="12"/>
       <c r="H46" s="12"/>
       <c r="I46" s="12"/>
-      <c r="J46" s="13" t="str">
-        <f aca="false">IF(COUNT(C46:I46)=0,"",SUM(C46:I46))</f>
-        <v/>
-      </c>
+      <c r="J46" s="12"/>
       <c r="K46" s="13" t="str">
-        <f aca="false">IF(B46="","",$J$5)</f>
+        <f aca="false">IF(COUNT(C46:J46)=0,"",SUM(C46:J46))</f>
         <v/>
       </c>
       <c r="L46" s="13" t="str">
-        <f aca="false">IF(J46="","",K46-J46)</f>
+        <f aca="false">IF(B46="","",$K$5)</f>
         <v/>
       </c>
       <c r="M46" s="13" t="str">
-        <f aca="false">IF(L46="","",SUM($L$10:L46))</f>
+        <f aca="false">IF(K46="","",L46-K46)</f>
+        <v/>
+      </c>
+      <c r="N46" s="13" t="str">
+        <f aca="false">IF(M46="","",SUM($M$10:M46))</f>
         <v/>
       </c>
     </row>
@@ -3176,7 +3294,7 @@
       <c r="A47" s="11" t="n">
         <v>38</v>
       </c>
-      <c r="B47" s="25" t="str">
+      <c r="B47" s="26" t="str">
         <f aca="false">IF(A47&gt;Budget!$B$7,"",Budget!$B$5+(A47-1)*7)</f>
         <v/>
       </c>
@@ -3187,20 +3305,21 @@
       <c r="G47" s="12"/>
       <c r="H47" s="12"/>
       <c r="I47" s="12"/>
-      <c r="J47" s="13" t="str">
-        <f aca="false">IF(COUNT(C47:I47)=0,"",SUM(C47:I47))</f>
-        <v/>
-      </c>
+      <c r="J47" s="12"/>
       <c r="K47" s="13" t="str">
-        <f aca="false">IF(B47="","",$J$5)</f>
+        <f aca="false">IF(COUNT(C47:J47)=0,"",SUM(C47:J47))</f>
         <v/>
       </c>
       <c r="L47" s="13" t="str">
-        <f aca="false">IF(J47="","",K47-J47)</f>
+        <f aca="false">IF(B47="","",$K$5)</f>
         <v/>
       </c>
       <c r="M47" s="13" t="str">
-        <f aca="false">IF(L47="","",SUM($L$10:L47))</f>
+        <f aca="false">IF(K47="","",L47-K47)</f>
+        <v/>
+      </c>
+      <c r="N47" s="13" t="str">
+        <f aca="false">IF(M47="","",SUM($M$10:M47))</f>
         <v/>
       </c>
     </row>
@@ -3208,7 +3327,7 @@
       <c r="A48" s="11" t="n">
         <v>39</v>
       </c>
-      <c r="B48" s="25" t="str">
+      <c r="B48" s="26" t="str">
         <f aca="false">IF(A48&gt;Budget!$B$7,"",Budget!$B$5+(A48-1)*7)</f>
         <v/>
       </c>
@@ -3219,20 +3338,21 @@
       <c r="G48" s="12"/>
       <c r="H48" s="12"/>
       <c r="I48" s="12"/>
-      <c r="J48" s="13" t="str">
-        <f aca="false">IF(COUNT(C48:I48)=0,"",SUM(C48:I48))</f>
-        <v/>
-      </c>
+      <c r="J48" s="12"/>
       <c r="K48" s="13" t="str">
-        <f aca="false">IF(B48="","",$J$5)</f>
+        <f aca="false">IF(COUNT(C48:J48)=0,"",SUM(C48:J48))</f>
         <v/>
       </c>
       <c r="L48" s="13" t="str">
-        <f aca="false">IF(J48="","",K48-J48)</f>
+        <f aca="false">IF(B48="","",$K$5)</f>
         <v/>
       </c>
       <c r="M48" s="13" t="str">
-        <f aca="false">IF(L48="","",SUM($L$10:L48))</f>
+        <f aca="false">IF(K48="","",L48-K48)</f>
+        <v/>
+      </c>
+      <c r="N48" s="13" t="str">
+        <f aca="false">IF(M48="","",SUM($M$10:M48))</f>
         <v/>
       </c>
     </row>
@@ -3240,7 +3360,7 @@
       <c r="A49" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="B49" s="25" t="str">
+      <c r="B49" s="26" t="str">
         <f aca="false">IF(A49&gt;Budget!$B$7,"",Budget!$B$5+(A49-1)*7)</f>
         <v/>
       </c>
@@ -3251,26 +3371,27 @@
       <c r="G49" s="12"/>
       <c r="H49" s="12"/>
       <c r="I49" s="12"/>
-      <c r="J49" s="13" t="str">
-        <f aca="false">IF(COUNT(C49:I49)=0,"",SUM(C49:I49))</f>
-        <v/>
-      </c>
+      <c r="J49" s="12"/>
       <c r="K49" s="13" t="str">
-        <f aca="false">IF(B49="","",$J$5)</f>
+        <f aca="false">IF(COUNT(C49:J49)=0,"",SUM(C49:J49))</f>
         <v/>
       </c>
       <c r="L49" s="13" t="str">
-        <f aca="false">IF(J49="","",K49-J49)</f>
+        <f aca="false">IF(B49="","",$K$5)</f>
         <v/>
       </c>
       <c r="M49" s="13" t="str">
-        <f aca="false">IF(L49="","",SUM($L$10:L49))</f>
+        <f aca="false">IF(K49="","",L49-K49)</f>
+        <v/>
+      </c>
+      <c r="N49" s="13" t="str">
+        <f aca="false">IF(M49="","",SUM($M$10:M49))</f>
         <v/>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B50" s="16"/>
       <c r="C50" s="17" t="n">
@@ -3305,74 +3426,82 @@
         <f aca="false">SUM(J10:J49)</f>
         <v>0</v>
       </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="17" t="n">
-        <f aca="false">SUM(L10:L49)</f>
+      <c r="K50" s="17" t="n">
+        <f aca="false">SUM(K10:K49)</f>
         <v>0</v>
       </c>
-      <c r="M50" s="16"/>
+      <c r="L50" s="16"/>
+      <c r="M50" s="17" t="n">
+        <f aca="false">SUM(M10:M49)</f>
+        <v>0</v>
+      </c>
+      <c r="N50" s="16"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="15" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B51" s="16"/>
       <c r="C51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",C50/COUNT(J10:J49))</f>
+        <f aca="false">IF(COUNT(K10:K49)=0,"",C50/COUNT(K10:K49))</f>
         <v/>
       </c>
       <c r="D51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",D50/COUNT(J10:J49))</f>
+        <f aca="false">IF(COUNT(K10:K49)=0,"",D50/COUNT(K10:K49))</f>
         <v/>
       </c>
       <c r="E51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",E50/COUNT(J10:J49))</f>
+        <f aca="false">IF(COUNT(K10:K49)=0,"",E50/COUNT(K10:K49))</f>
         <v/>
       </c>
       <c r="F51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",F50/COUNT(J10:J49))</f>
+        <f aca="false">IF(COUNT(K10:K49)=0,"",F50/COUNT(K10:K49))</f>
         <v/>
       </c>
       <c r="G51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",G50/COUNT(J10:J49))</f>
+        <f aca="false">IF(COUNT(K10:K49)=0,"",G50/COUNT(K10:K49))</f>
         <v/>
       </c>
       <c r="H51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",H50/COUNT(J10:J49))</f>
+        <f aca="false">IF(COUNT(K10:K49)=0,"",H50/COUNT(K10:K49))</f>
         <v/>
       </c>
       <c r="I51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",I50/COUNT(J10:J49))</f>
+        <f aca="false">IF(COUNT(K10:K49)=0,"",I50/COUNT(K10:K49))</f>
         <v/>
       </c>
       <c r="J51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",J50/COUNT(J10:J49))</f>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="17" t="str">
-        <f aca="false">IF(COUNT(J10:J49)=0,"",L50/COUNT(J10:J49))</f>
-        <v/>
-      </c>
-      <c r="M51" s="16"/>
+        <f aca="false">IF(COUNT(K10:K49)=0,"",J50/COUNT(K10:K49))</f>
+        <v/>
+      </c>
+      <c r="K51" s="17" t="str">
+        <f aca="false">IF(COUNT(K10:K49)=0,"",K50/COUNT(K10:K49))</f>
+        <v/>
+      </c>
+      <c r="L51" s="16"/>
+      <c r="M51" s="17" t="str">
+        <f aca="false">IF(COUNT(K10:K49)=0,"",M50/COUNT(K10:K49))</f>
+        <v/>
+      </c>
+      <c r="N51" s="16"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C10:I49">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+  <conditionalFormatting sqref="C10:J49">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>AND(ISNUMBER(C10),C10&gt;C$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C51:I51">
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+  <conditionalFormatting sqref="C51:J51">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>AND(ISNUMBER(C51),C51&gt;C$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L10:M49">
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>AND(ISNUMBER(L10),L10&lt;0)</formula>
+  <conditionalFormatting sqref="M10:N49">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND(ISNUMBER(M10),M10&lt;0)</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>AND(ISNUMBER(L10),L10&gt;=0)</formula>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>AND(ISNUMBER(M10),M10&gt;=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3390,7 +3519,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -3398,126 +3527,134 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>90</v>
+      <c r="A3" s="27" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
-        <v>92</v>
+      <c r="A4" s="28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="28" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27"/>
+      <c r="A6" s="28"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="27" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="28" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="27" t="s">
-        <v>96</v>
+      <c r="A10" s="28" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="s">
-        <v>97</v>
-      </c>
+      <c r="A11" s="28"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="27"/>
+      <c r="A13" s="28" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="26" t="s">
-        <v>99</v>
+      <c r="A14" s="28" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="27" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="28"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="27" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="27" t="s">
         <v>103</v>
       </c>
     </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="28" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="28" t="s">
+        <v>105</v>
+      </c>
+    </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="27" t="s">
-        <v>104</v>
+      <c r="A19" s="28" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="27" t="s">
-        <v>105</v>
+      <c r="A20" s="28" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="27" t="s">
-        <v>106</v>
+      <c r="A21" s="28" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="27" t="s">
-        <v>107</v>
+      <c r="A22" s="28" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27"/>
+      <c r="A23" s="28" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26" t="s">
-        <v>108</v>
-      </c>
+      <c r="A24" s="28"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="27" t="s">
-        <v>110</v>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="28" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="27" t="s">
-        <v>111</v>
+      <c r="A27" s="28" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="28" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>